<commit_message>
feat: Add new slides and data for '뉴 이재명' analysis; update chart utilities and slide rendering logic fix: Corrected data formatting in line chart and updated settings for script execution delete: Remove outdated Excel file related to previous analysis
</commit_message>
<xml_diff>
--- a/2603newjm/그래프_수정.xlsx
+++ b/2603newjm/그래프_수정.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goodsti.sharepoint.com/sites/2026/Shared Documents/2026 정당학회-한겨레 패널조사 (4-5차)/토론회/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\WeeklyOpinion\2603newjm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="552" documentId="13_ncr:1_{E426FD80-5845-4265-B6A7-AF2E458DD5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EE85204-276D-4051-B72E-4AE0E2130C07}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E8F5B9-9276-4D4A-8C3B-F4B532B8BDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30030" yWindow="1335" windowWidth="27330" windowHeight="13380" tabRatio="771" activeTab="10" xr2:uid="{E410F4C7-6FD6-4BE3-A662-B6CB9E02DB3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="771" activeTab="4" xr2:uid="{E410F4C7-6FD6-4BE3-A662-B6CB9E02DB3D}"/>
   </bookViews>
   <sheets>
     <sheet name="4p" sheetId="1" r:id="rId1"/>
@@ -1833,7 +1833,7 @@
     <numFmt numFmtId="179" formatCode="0.0_ "/>
     <numFmt numFmtId="180" formatCode="0_ "/>
     <numFmt numFmtId="181" formatCode="0.0_);[Red]\(0.0\)"/>
-    <numFmt numFmtId="189" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="182" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -3536,177 +3536,6 @@
     <xf numFmtId="176" fontId="20" fillId="7" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="49" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3717,30 +3546,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3755,9 +3560,6 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3767,22 +3569,16 @@
     <xf numFmtId="176" fontId="10" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="189" fontId="29" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="29" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3824,10 +3620,142 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="10" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3845,17 +3773,89 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="40" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="49" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -11895,7 +11895,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ko-KR"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -31783,33 +31783,33 @@
   <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="176" t="s">
+      <c r="A1" s="214" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="176" t="s">
+      <c r="B1" s="214" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="176" t="s">
+      <c r="C1" s="214" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="176" t="s">
+      <c r="D1" s="214" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="6"/>
-      <c r="F1" s="171" t="s">
+      <c r="F1" s="205" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="172"/>
-      <c r="H1" s="172"/>
-      <c r="I1" s="172"/>
-      <c r="J1" s="172"/>
-      <c r="K1" s="173"/>
+      <c r="G1" s="206"/>
+      <c r="H1" s="206"/>
+      <c r="I1" s="206"/>
+      <c r="J1" s="206"/>
+      <c r="K1" s="207"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="177"/>
-      <c r="B2" s="177"/>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
+      <c r="A2" s="215"/>
+      <c r="B2" s="215"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
       <c r="E2" s="3"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
@@ -31831,7 +31831,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="25.5">
-      <c r="A3" s="176" t="s">
+      <c r="A3" s="214" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -31866,7 +31866,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="25.5">
-      <c r="A4" s="177"/>
+      <c r="A4" s="215"/>
       <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
@@ -31910,7 +31910,7 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="25.5">
-      <c r="A18" s="174" t="s">
+      <c r="A18" s="208" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -31936,7 +31936,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="25.5">
-      <c r="A19" s="175"/>
+      <c r="A19" s="209"/>
       <c r="B19" s="4" t="s">
         <v>14</v>
       </c>
@@ -31960,42 +31960,42 @@
       </c>
     </row>
     <row r="36" spans="3:11">
-      <c r="C36" s="169"/>
-      <c r="D36" s="165" t="s">
+      <c r="C36" s="212"/>
+      <c r="D36" s="210" t="s">
         <v>33</v>
       </c>
-      <c r="E36" s="165" t="s">
+      <c r="E36" s="210" t="s">
         <v>27</v>
       </c>
-      <c r="F36" s="165" t="s">
+      <c r="F36" s="210" t="s">
         <v>28</v>
       </c>
-      <c r="G36" s="165" t="s">
+      <c r="G36" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="H36" s="165" t="s">
+      <c r="H36" s="210" t="s">
         <v>30</v>
       </c>
-      <c r="I36" s="165" t="s">
+      <c r="I36" s="210" t="s">
         <v>31</v>
       </c>
-      <c r="J36" s="165" t="s">
+      <c r="J36" s="210" t="s">
         <v>9</v>
       </c>
-      <c r="K36" s="165" t="s">
+      <c r="K36" s="210" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="37" spans="3:11">
-      <c r="C37" s="170"/>
-      <c r="D37" s="166"/>
-      <c r="E37" s="166"/>
-      <c r="F37" s="166"/>
-      <c r="G37" s="166"/>
-      <c r="H37" s="166"/>
-      <c r="I37" s="166"/>
-      <c r="J37" s="166"/>
-      <c r="K37" s="166"/>
+      <c r="C37" s="213"/>
+      <c r="D37" s="211"/>
+      <c r="E37" s="211"/>
+      <c r="F37" s="211"/>
+      <c r="G37" s="211"/>
+      <c r="H37" s="211"/>
+      <c r="I37" s="211"/>
+      <c r="J37" s="211"/>
+      <c r="K37" s="211"/>
     </row>
     <row r="38" spans="3:11" ht="25.5">
       <c r="C38" s="2" t="s">
@@ -32174,46 +32174,46 @@
       </c>
     </row>
     <row r="96" spans="4:14" ht="16.5" customHeight="1">
-      <c r="D96" s="167"/>
-      <c r="E96" s="167"/>
-      <c r="F96" s="169"/>
-      <c r="G96" s="165" t="s">
+      <c r="D96" s="216"/>
+      <c r="E96" s="216"/>
+      <c r="F96" s="212"/>
+      <c r="G96" s="210" t="s">
         <v>33</v>
       </c>
-      <c r="H96" s="165" t="s">
+      <c r="H96" s="210" t="s">
         <v>27</v>
       </c>
-      <c r="I96" s="165" t="s">
+      <c r="I96" s="210" t="s">
         <v>28</v>
       </c>
-      <c r="J96" s="165" t="s">
+      <c r="J96" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="K96" s="165" t="s">
+      <c r="K96" s="210" t="s">
         <v>30</v>
       </c>
-      <c r="L96" s="165" t="s">
+      <c r="L96" s="210" t="s">
         <v>31</v>
       </c>
-      <c r="M96" s="165" t="s">
+      <c r="M96" s="210" t="s">
         <v>9</v>
       </c>
-      <c r="N96" s="165" t="s">
+      <c r="N96" s="210" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="97" spans="4:14" ht="16.5" customHeight="1">
-      <c r="D97" s="168"/>
-      <c r="E97" s="168"/>
-      <c r="F97" s="170"/>
-      <c r="G97" s="166"/>
-      <c r="H97" s="166"/>
-      <c r="I97" s="166"/>
-      <c r="J97" s="166"/>
-      <c r="K97" s="166"/>
-      <c r="L97" s="166"/>
-      <c r="M97" s="166"/>
-      <c r="N97" s="166"/>
+      <c r="D97" s="217"/>
+      <c r="E97" s="217"/>
+      <c r="F97" s="213"/>
+      <c r="G97" s="211"/>
+      <c r="H97" s="211"/>
+      <c r="I97" s="211"/>
+      <c r="J97" s="211"/>
+      <c r="K97" s="211"/>
+      <c r="L97" s="211"/>
+      <c r="M97" s="211"/>
+      <c r="N97" s="211"/>
     </row>
     <row r="98" spans="4:14">
       <c r="D98" s="12" t="s">
@@ -32320,49 +32320,49 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="122" spans="4:14" ht="16.5" customHeight="1">
-      <c r="D122" s="167"/>
-      <c r="E122" s="167"/>
-      <c r="F122" s="169"/>
-      <c r="G122" s="165" t="s">
+    <row r="122" spans="4:16" ht="16.5" customHeight="1">
+      <c r="D122" s="216"/>
+      <c r="E122" s="216"/>
+      <c r="F122" s="212"/>
+      <c r="G122" s="210" t="s">
         <v>33</v>
       </c>
-      <c r="H122" s="165" t="s">
+      <c r="H122" s="210" t="s">
         <v>27</v>
       </c>
-      <c r="I122" s="165" t="s">
+      <c r="I122" s="210" t="s">
         <v>28</v>
       </c>
-      <c r="J122" s="165" t="s">
+      <c r="J122" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="K122" s="165" t="s">
+      <c r="K122" s="210" t="s">
         <v>30</v>
       </c>
-      <c r="L122" s="165" t="s">
+      <c r="L122" s="210" t="s">
         <v>31</v>
       </c>
-      <c r="M122" s="165" t="s">
+      <c r="M122" s="210" t="s">
         <v>9</v>
       </c>
-      <c r="N122" s="165" t="s">
+      <c r="N122" s="210" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="4:14" ht="16.5" customHeight="1">
-      <c r="D123" s="168"/>
-      <c r="E123" s="168"/>
-      <c r="F123" s="170"/>
-      <c r="G123" s="166"/>
-      <c r="H123" s="166"/>
-      <c r="I123" s="166"/>
-      <c r="J123" s="166"/>
-      <c r="K123" s="166"/>
-      <c r="L123" s="166"/>
-      <c r="M123" s="166"/>
-      <c r="N123" s="166"/>
+    <row r="123" spans="4:16" ht="16.5" customHeight="1">
+      <c r="D123" s="217"/>
+      <c r="E123" s="217"/>
+      <c r="F123" s="213"/>
+      <c r="G123" s="211"/>
+      <c r="H123" s="211"/>
+      <c r="I123" s="211"/>
+      <c r="J123" s="211"/>
+      <c r="K123" s="211"/>
+      <c r="L123" s="211"/>
+      <c r="M123" s="211"/>
+      <c r="N123" s="211"/>
     </row>
-    <row r="124" spans="4:14">
+    <row r="124" spans="4:16">
       <c r="D124" s="12"/>
       <c r="E124" s="12"/>
       <c r="F124" t="s">
@@ -32392,8 +32392,12 @@
       <c r="N124" s="13">
         <v>0.8</v>
       </c>
+      <c r="P124">
+        <f>SUM(J124,L124,M124,N124)</f>
+        <v>5.3</v>
+      </c>
     </row>
-    <row r="125" spans="4:14">
+    <row r="125" spans="4:16">
       <c r="F125" t="s">
         <v>42</v>
       </c>
@@ -32420,6 +32424,10 @@
       </c>
       <c r="N125" s="13">
         <v>4.8</v>
+      </c>
+      <c r="P125">
+        <f>SUM(J125,L125,M125,N125)</f>
+        <v>23.6</v>
       </c>
     </row>
     <row r="130" spans="18:18">
@@ -32429,6 +32437,28 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="K122:K123"/>
+    <mergeCell ref="M122:M123"/>
+    <mergeCell ref="N122:N123"/>
+    <mergeCell ref="G122:G123"/>
+    <mergeCell ref="L122:L123"/>
+    <mergeCell ref="K96:K97"/>
+    <mergeCell ref="M96:M97"/>
+    <mergeCell ref="N96:N97"/>
+    <mergeCell ref="G96:G97"/>
+    <mergeCell ref="L96:L97"/>
+    <mergeCell ref="J96:J97"/>
+    <mergeCell ref="J122:J123"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="F96:F97"/>
+    <mergeCell ref="H96:H97"/>
+    <mergeCell ref="I96:I97"/>
+    <mergeCell ref="D122:D123"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="F122:F123"/>
+    <mergeCell ref="H122:H123"/>
+    <mergeCell ref="I122:I123"/>
     <mergeCell ref="F1:K1"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="E36:E37"/>
@@ -32445,28 +32475,6 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="J36:J37"/>
-    <mergeCell ref="D122:D123"/>
-    <mergeCell ref="E122:E123"/>
-    <mergeCell ref="F122:F123"/>
-    <mergeCell ref="H122:H123"/>
-    <mergeCell ref="I122:I123"/>
-    <mergeCell ref="J122:J123"/>
-    <mergeCell ref="D96:D97"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="F96:F97"/>
-    <mergeCell ref="H96:H97"/>
-    <mergeCell ref="I96:I97"/>
-    <mergeCell ref="K96:K97"/>
-    <mergeCell ref="M96:M97"/>
-    <mergeCell ref="N96:N97"/>
-    <mergeCell ref="G96:G97"/>
-    <mergeCell ref="L96:L97"/>
-    <mergeCell ref="J96:J97"/>
-    <mergeCell ref="K122:K123"/>
-    <mergeCell ref="M122:M123"/>
-    <mergeCell ref="N122:N123"/>
-    <mergeCell ref="G122:G123"/>
-    <mergeCell ref="L122:L123"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -32870,50 +32878,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.25" thickTop="1">
-      <c r="B1" s="226"/>
-      <c r="C1" s="228" t="s">
+      <c r="B1" s="197"/>
+      <c r="C1" s="203" t="s">
         <v>245</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>246</v>
       </c>
-      <c r="E1" s="228" t="s">
+      <c r="E1" s="203" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="228" t="s">
+      <c r="F1" s="203" t="s">
         <v>71</v>
       </c>
       <c r="G1" s="16" t="s">
         <v>246</v>
       </c>
-      <c r="H1" s="230" t="s">
+      <c r="H1" s="199" t="s">
         <v>247</v>
       </c>
-      <c r="I1" s="230" t="s">
+      <c r="I1" s="199" t="s">
         <v>248</v>
       </c>
-      <c r="J1" s="232" t="s">
+      <c r="J1" s="201" t="s">
         <v>249</v>
       </c>
-      <c r="K1" s="232" t="s">
+      <c r="K1" s="201" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="17.25" thickBot="1">
-      <c r="B2" s="227"/>
-      <c r="C2" s="229"/>
-      <c r="D2" s="222" t="s">
+      <c r="B2" s="198"/>
+      <c r="C2" s="204"/>
+      <c r="D2" s="165" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="229"/>
-      <c r="F2" s="229"/>
-      <c r="G2" s="222" t="s">
+      <c r="E2" s="204"/>
+      <c r="F2" s="204"/>
+      <c r="G2" s="165" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="231"/>
-      <c r="I2" s="231"/>
-      <c r="J2" s="233"/>
-      <c r="K2" s="233"/>
+      <c r="H2" s="200"/>
+      <c r="I2" s="200"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
     </row>
     <row r="3" spans="1:11" ht="17.25" thickTop="1">
       <c r="A3" t="s">
@@ -32937,16 +32945,16 @@
       <c r="G3" s="48">
         <v>1.6</v>
       </c>
-      <c r="H3" s="234">
+      <c r="H3" s="169">
         <v>79.900000000000006</v>
       </c>
-      <c r="I3" s="234">
+      <c r="I3" s="169">
         <v>20.100000000000001</v>
       </c>
-      <c r="J3" s="235">
+      <c r="J3" s="170">
         <v>2</v>
       </c>
-      <c r="K3" s="235">
+      <c r="K3" s="170">
         <v>0.67</v>
       </c>
     </row>
@@ -32969,16 +32977,16 @@
       <c r="G4" s="44">
         <v>5.2</v>
       </c>
-      <c r="H4" s="236">
+      <c r="H4" s="171">
         <v>59.1</v>
       </c>
-      <c r="I4" s="236">
+      <c r="I4" s="171">
         <v>40.9</v>
       </c>
-      <c r="J4" s="237">
+      <c r="J4" s="172">
         <v>2.4</v>
       </c>
-      <c r="K4" s="237">
+      <c r="K4" s="172">
         <v>0.73</v>
       </c>
     </row>
@@ -33004,16 +33012,16 @@
       <c r="G5" s="48">
         <v>2</v>
       </c>
-      <c r="H5" s="234">
+      <c r="H5" s="169">
         <v>89.1</v>
       </c>
-      <c r="I5" s="234">
+      <c r="I5" s="169">
         <v>10.9</v>
       </c>
-      <c r="J5" s="235">
+      <c r="J5" s="170">
         <v>1.7</v>
       </c>
-      <c r="K5" s="235">
+      <c r="K5" s="170">
         <v>0.7</v>
       </c>
     </row>
@@ -33036,16 +33044,16 @@
       <c r="G6" s="44">
         <v>5.3</v>
       </c>
-      <c r="H6" s="236">
+      <c r="H6" s="171">
         <v>64.900000000000006</v>
       </c>
-      <c r="I6" s="236">
+      <c r="I6" s="171">
         <v>35.1</v>
       </c>
-      <c r="J6" s="237">
+      <c r="J6" s="172">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K6" s="237">
+      <c r="K6" s="172">
         <v>0.79</v>
       </c>
     </row>
@@ -33071,16 +33079,16 @@
       <c r="G7" s="48">
         <v>2.2000000000000002</v>
       </c>
-      <c r="H7" s="234">
+      <c r="H7" s="169">
         <v>75.5</v>
       </c>
-      <c r="I7" s="234">
+      <c r="I7" s="169">
         <v>24.5</v>
       </c>
-      <c r="J7" s="235">
+      <c r="J7" s="170">
         <v>2.1</v>
       </c>
-      <c r="K7" s="235">
+      <c r="K7" s="170">
         <v>0.71</v>
       </c>
     </row>
@@ -33103,16 +33111,16 @@
       <c r="G8" s="44">
         <v>10</v>
       </c>
-      <c r="H8" s="236">
+      <c r="H8" s="171">
         <v>46.9</v>
       </c>
-      <c r="I8" s="236">
+      <c r="I8" s="171">
         <v>53.1</v>
       </c>
-      <c r="J8" s="237">
+      <c r="J8" s="172">
         <v>2.6</v>
       </c>
-      <c r="K8" s="237">
+      <c r="K8" s="172">
         <v>0.78</v>
       </c>
     </row>
@@ -33138,16 +33146,16 @@
       <c r="G9" s="48">
         <v>10.7</v>
       </c>
-      <c r="H9" s="234">
+      <c r="H9" s="169">
         <v>55</v>
       </c>
-      <c r="I9" s="234">
+      <c r="I9" s="169">
         <v>45</v>
       </c>
-      <c r="J9" s="235">
+      <c r="J9" s="170">
         <v>2.4</v>
       </c>
-      <c r="K9" s="235">
+      <c r="K9" s="170">
         <v>0.87</v>
       </c>
     </row>
@@ -33170,16 +33178,16 @@
       <c r="G10" s="44">
         <v>8</v>
       </c>
-      <c r="H10" s="236">
+      <c r="H10" s="171">
         <v>65.3</v>
       </c>
-      <c r="I10" s="236">
+      <c r="I10" s="171">
         <v>34.700000000000003</v>
       </c>
-      <c r="J10" s="237">
+      <c r="J10" s="172">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K10" s="237">
+      <c r="K10" s="172">
         <v>0.85</v>
       </c>
     </row>
@@ -33205,16 +33213,16 @@
       <c r="G11" s="48">
         <v>16.100000000000001</v>
       </c>
-      <c r="H11" s="234">
+      <c r="H11" s="169">
         <v>21</v>
       </c>
-      <c r="I11" s="234">
+      <c r="I11" s="169">
         <v>79</v>
       </c>
-      <c r="J11" s="235">
+      <c r="J11" s="170">
         <v>2.9</v>
       </c>
-      <c r="K11" s="235">
+      <c r="K11" s="170">
         <v>0.65</v>
       </c>
     </row>
@@ -33237,16 +33245,16 @@
       <c r="G12" s="44">
         <v>10.6</v>
       </c>
-      <c r="H12" s="236">
+      <c r="H12" s="171">
         <v>33.6</v>
       </c>
-      <c r="I12" s="236">
+      <c r="I12" s="171">
         <v>66.400000000000006</v>
       </c>
-      <c r="J12" s="237">
+      <c r="J12" s="172">
         <v>2.7</v>
       </c>
-      <c r="K12" s="237">
+      <c r="K12" s="172">
         <v>0.67</v>
       </c>
     </row>
@@ -33272,16 +33280,16 @@
       <c r="G13" s="48">
         <v>4</v>
       </c>
-      <c r="H13" s="234">
+      <c r="H13" s="169">
         <v>81.8</v>
       </c>
-      <c r="I13" s="234">
+      <c r="I13" s="169">
         <v>18.2</v>
       </c>
-      <c r="J13" s="235">
+      <c r="J13" s="170">
         <v>2</v>
       </c>
-      <c r="K13" s="235">
+      <c r="K13" s="170">
         <v>0.69</v>
       </c>
     </row>
@@ -33304,71 +33312,71 @@
       <c r="G14" s="44">
         <v>14.8</v>
       </c>
-      <c r="H14" s="236">
+      <c r="H14" s="171">
         <v>59.8</v>
       </c>
-      <c r="I14" s="236">
+      <c r="I14" s="171">
         <v>40.200000000000003</v>
       </c>
-      <c r="J14" s="237">
+      <c r="J14" s="172">
         <v>2.5</v>
       </c>
-      <c r="K14" s="237">
+      <c r="K14" s="172">
         <v>0.86</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="17.25" thickBot="1"/>
     <row r="20" spans="1:13" ht="17.25" thickTop="1">
-      <c r="A20" s="238"/>
-      <c r="B20" s="226"/>
-      <c r="C20" s="230" t="s">
+      <c r="A20" s="195"/>
+      <c r="B20" s="197"/>
+      <c r="C20" s="199" t="s">
         <v>247</v>
       </c>
-      <c r="D20" s="230" t="s">
+      <c r="D20" s="199" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A21" s="238"/>
-      <c r="B21" s="227"/>
-      <c r="C21" s="231"/>
-      <c r="D21" s="231"/>
-      <c r="J21" s="244" t="s">
+      <c r="A21" s="195"/>
+      <c r="B21" s="198"/>
+      <c r="C21" s="200"/>
+      <c r="D21" s="200"/>
+      <c r="J21" s="177" t="s">
         <v>257</v>
       </c>
-      <c r="K21" s="244" t="s">
+      <c r="K21" s="177" t="s">
         <v>258</v>
       </c>
-      <c r="L21" s="244" t="s">
+      <c r="L21" s="177" t="s">
         <v>259</v>
       </c>
-      <c r="M21" s="244" t="s">
+      <c r="M21" s="177" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A22" s="239" t="s">
+      <c r="A22" s="196" t="s">
         <v>251</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="240">
+      <c r="C22" s="174">
         <v>79.900000000000006</v>
       </c>
-      <c r="D22" s="240">
+      <c r="D22" s="174">
         <v>20.100000000000001</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="241">
+      <c r="F22" s="175">
         <v>59.1</v>
       </c>
-      <c r="G22" s="241">
+      <c r="G22" s="175">
         <v>40.9</v>
       </c>
-      <c r="J22" s="245" t="s">
+      <c r="J22" s="194" t="s">
         <v>251</v>
       </c>
       <c r="K22" s="139" t="s">
@@ -33382,26 +33390,26 @@
       </c>
     </row>
     <row r="23" spans="1:13" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A23" s="239"/>
+      <c r="A23" s="196"/>
       <c r="B23" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="241">
+      <c r="C23" s="175">
         <v>59.1</v>
       </c>
-      <c r="D23" s="241">
+      <c r="D23" s="175">
         <v>40.9</v>
       </c>
       <c r="E23" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="240">
+      <c r="F23" s="174">
         <v>79.900000000000006</v>
       </c>
-      <c r="G23" s="240">
+      <c r="G23" s="174">
         <v>20.100000000000001</v>
       </c>
-      <c r="J23" s="245"/>
+      <c r="J23" s="194"/>
       <c r="K23" s="139" t="s">
         <v>47</v>
       </c>
@@ -33413,26 +33421,26 @@
       </c>
     </row>
     <row r="24" spans="1:13" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A24" s="242"/>
-      <c r="B24" s="243" t="s">
+      <c r="A24" s="173"/>
+      <c r="B24" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C24" s="224">
+      <c r="C24" s="167">
         <v>60.4</v>
       </c>
-      <c r="D24" s="224">
+      <c r="D24" s="167">
         <v>39.6</v>
       </c>
-      <c r="E24" s="243" t="s">
+      <c r="E24" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F24" s="224">
+      <c r="F24" s="167">
         <v>60.4</v>
       </c>
-      <c r="G24" s="224">
+      <c r="G24" s="167">
         <v>39.6</v>
       </c>
-      <c r="J24" s="245"/>
+      <c r="J24" s="194"/>
       <c r="K24" s="139" t="s">
         <v>151</v>
       </c>
@@ -33444,28 +33452,28 @@
       </c>
     </row>
     <row r="25" spans="1:13" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A25" s="239" t="s">
+      <c r="A25" s="196" t="s">
         <v>252</v>
       </c>
       <c r="B25" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="240">
+      <c r="C25" s="174">
         <v>89.1</v>
       </c>
-      <c r="D25" s="240">
+      <c r="D25" s="174">
         <v>10.9</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="241">
+      <c r="F25" s="175">
         <v>64.900000000000006</v>
       </c>
-      <c r="G25" s="241">
+      <c r="G25" s="175">
         <v>35.1</v>
       </c>
-      <c r="J25" s="245" t="s">
+      <c r="J25" s="194" t="s">
         <v>252</v>
       </c>
       <c r="K25" s="139" t="s">
@@ -33479,26 +33487,26 @@
       </c>
     </row>
     <row r="26" spans="1:13" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A26" s="239"/>
+      <c r="A26" s="196"/>
       <c r="B26" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="241">
+      <c r="C26" s="175">
         <v>64.900000000000006</v>
       </c>
-      <c r="D26" s="241">
+      <c r="D26" s="175">
         <v>35.1</v>
       </c>
       <c r="E26" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="240">
+      <c r="F26" s="174">
         <v>89.1</v>
       </c>
-      <c r="G26" s="240">
+      <c r="G26" s="174">
         <v>10.9</v>
       </c>
-      <c r="J26" s="245"/>
+      <c r="J26" s="194"/>
       <c r="K26" s="139" t="s">
         <v>47</v>
       </c>
@@ -33510,26 +33518,26 @@
       </c>
     </row>
     <row r="27" spans="1:13" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A27" s="242"/>
-      <c r="B27" s="243" t="s">
+      <c r="A27" s="173"/>
+      <c r="B27" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C27" s="224">
+      <c r="C27" s="167">
         <v>68.8</v>
       </c>
-      <c r="D27" s="224">
+      <c r="D27" s="167">
         <v>31.2</v>
       </c>
-      <c r="E27" s="243" t="s">
+      <c r="E27" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F27" s="224">
+      <c r="F27" s="167">
         <v>68.8</v>
       </c>
-      <c r="G27" s="224">
+      <c r="G27" s="167">
         <v>31.2</v>
       </c>
-      <c r="J27" s="245"/>
+      <c r="J27" s="194"/>
       <c r="K27" s="139" t="s">
         <v>151</v>
       </c>
@@ -33541,28 +33549,28 @@
       </c>
     </row>
     <row r="28" spans="1:13" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A28" s="239" t="s">
+      <c r="A28" s="196" t="s">
         <v>253</v>
       </c>
       <c r="B28" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="240">
+      <c r="C28" s="174">
         <v>75.5</v>
       </c>
-      <c r="D28" s="240">
+      <c r="D28" s="174">
         <v>24.5</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F28" s="241">
+      <c r="F28" s="175">
         <v>46.9</v>
       </c>
-      <c r="G28" s="241">
+      <c r="G28" s="175">
         <v>53.1</v>
       </c>
-      <c r="J28" s="245" t="s">
+      <c r="J28" s="194" t="s">
         <v>253</v>
       </c>
       <c r="K28" s="139" t="s">
@@ -33576,26 +33584,26 @@
       </c>
     </row>
     <row r="29" spans="1:13" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A29" s="239"/>
+      <c r="A29" s="196"/>
       <c r="B29" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="241">
+      <c r="C29" s="175">
         <v>46.9</v>
       </c>
-      <c r="D29" s="241">
+      <c r="D29" s="175">
         <v>53.1</v>
       </c>
       <c r="E29" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F29" s="240">
+      <c r="F29" s="174">
         <v>75.5</v>
       </c>
-      <c r="G29" s="240">
+      <c r="G29" s="174">
         <v>24.5</v>
       </c>
-      <c r="J29" s="245"/>
+      <c r="J29" s="194"/>
       <c r="K29" s="139" t="s">
         <v>47</v>
       </c>
@@ -33607,26 +33615,26 @@
       </c>
     </row>
     <row r="30" spans="1:13" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A30" s="242"/>
-      <c r="B30" s="243" t="s">
+      <c r="A30" s="173"/>
+      <c r="B30" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C30" s="224">
+      <c r="C30" s="167">
         <v>53.3</v>
       </c>
-      <c r="D30" s="224">
+      <c r="D30" s="167">
         <v>46.7</v>
       </c>
-      <c r="E30" s="243" t="s">
+      <c r="E30" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F30" s="224">
+      <c r="F30" s="167">
         <v>53.3</v>
       </c>
-      <c r="G30" s="224">
+      <c r="G30" s="167">
         <v>46.7</v>
       </c>
-      <c r="J30" s="245"/>
+      <c r="J30" s="194"/>
       <c r="K30" s="139" t="s">
         <v>151</v>
       </c>
@@ -33638,28 +33646,28 @@
       </c>
     </row>
     <row r="31" spans="1:13" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A31" s="239" t="s">
+      <c r="A31" s="196" t="s">
         <v>254</v>
       </c>
       <c r="B31" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="240">
+      <c r="C31" s="174">
         <v>55</v>
       </c>
-      <c r="D31" s="240">
+      <c r="D31" s="174">
         <v>45</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F31" s="241">
+      <c r="F31" s="175">
         <v>65.3</v>
       </c>
-      <c r="G31" s="241">
+      <c r="G31" s="175">
         <v>34.700000000000003</v>
       </c>
-      <c r="J31" s="245" t="s">
+      <c r="J31" s="194" t="s">
         <v>254</v>
       </c>
       <c r="K31" s="139" t="s">
@@ -33673,26 +33681,26 @@
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A32" s="239"/>
+      <c r="A32" s="196"/>
       <c r="B32" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="241">
+      <c r="C32" s="175">
         <v>65.3</v>
       </c>
-      <c r="D32" s="241">
+      <c r="D32" s="175">
         <v>34.700000000000003</v>
       </c>
       <c r="E32" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F32" s="240">
+      <c r="F32" s="174">
         <v>55</v>
       </c>
-      <c r="G32" s="240">
+      <c r="G32" s="174">
         <v>45</v>
       </c>
-      <c r="J32" s="245"/>
+      <c r="J32" s="194"/>
       <c r="K32" s="139" t="s">
         <v>47</v>
       </c>
@@ -33704,26 +33712,26 @@
       </c>
     </row>
     <row r="33" spans="1:15" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A33" s="242"/>
-      <c r="B33" s="243" t="s">
+      <c r="A33" s="173"/>
+      <c r="B33" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C33" s="224">
+      <c r="C33" s="167">
         <v>65.2</v>
       </c>
-      <c r="D33" s="224">
+      <c r="D33" s="167">
         <v>34.799999999999997</v>
       </c>
-      <c r="E33" s="243" t="s">
+      <c r="E33" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F33" s="224">
+      <c r="F33" s="167">
         <v>65.2</v>
       </c>
-      <c r="G33" s="224">
+      <c r="G33" s="167">
         <v>34.799999999999997</v>
       </c>
-      <c r="J33" s="245"/>
+      <c r="J33" s="194"/>
       <c r="K33" s="139" t="s">
         <v>151</v>
       </c>
@@ -33735,28 +33743,28 @@
       </c>
     </row>
     <row r="34" spans="1:15" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A34" s="239" t="s">
+      <c r="A34" s="196" t="s">
         <v>255</v>
       </c>
       <c r="B34" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="240">
+      <c r="C34" s="174">
         <v>21</v>
       </c>
-      <c r="D34" s="240">
+      <c r="D34" s="174">
         <v>79</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F34" s="241">
+      <c r="F34" s="175">
         <v>33.6</v>
       </c>
-      <c r="G34" s="241">
+      <c r="G34" s="175">
         <v>66.400000000000006</v>
       </c>
-      <c r="J34" s="245" t="s">
+      <c r="J34" s="194" t="s">
         <v>255</v>
       </c>
       <c r="K34" s="139" t="s">
@@ -33770,26 +33778,26 @@
       </c>
     </row>
     <row r="35" spans="1:15" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A35" s="239"/>
+      <c r="A35" s="196"/>
       <c r="B35" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="241">
+      <c r="C35" s="175">
         <v>33.6</v>
       </c>
-      <c r="D35" s="241">
+      <c r="D35" s="175">
         <v>66.400000000000006</v>
       </c>
       <c r="E35" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F35" s="240">
+      <c r="F35" s="174">
         <v>21</v>
       </c>
-      <c r="G35" s="240">
+      <c r="G35" s="174">
         <v>79</v>
       </c>
-      <c r="J35" s="245"/>
+      <c r="J35" s="194"/>
       <c r="K35" s="139" t="s">
         <v>47</v>
       </c>
@@ -33801,26 +33809,26 @@
       </c>
     </row>
     <row r="36" spans="1:15" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A36" s="242"/>
-      <c r="B36" s="243" t="s">
+      <c r="A36" s="173"/>
+      <c r="B36" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C36" s="224">
+      <c r="C36" s="167">
         <v>35.4</v>
       </c>
-      <c r="D36" s="224">
+      <c r="D36" s="167">
         <v>64.599999999999994</v>
       </c>
-      <c r="E36" s="243" t="s">
+      <c r="E36" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F36" s="224">
+      <c r="F36" s="167">
         <v>35.4</v>
       </c>
-      <c r="G36" s="224">
+      <c r="G36" s="167">
         <v>64.599999999999994</v>
       </c>
-      <c r="J36" s="245"/>
+      <c r="J36" s="194"/>
       <c r="K36" s="139" t="s">
         <v>151</v>
       </c>
@@ -33832,28 +33840,28 @@
       </c>
     </row>
     <row r="37" spans="1:15" ht="15.6" customHeight="1" thickTop="1">
-      <c r="A37" s="239" t="s">
+      <c r="A37" s="196" t="s">
         <v>256</v>
       </c>
       <c r="B37" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C37" s="240">
+      <c r="C37" s="174">
         <v>81.8</v>
       </c>
-      <c r="D37" s="240">
+      <c r="D37" s="174">
         <v>18.2</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F37" s="241">
+      <c r="F37" s="175">
         <v>59.8</v>
       </c>
-      <c r="G37" s="241">
+      <c r="G37" s="175">
         <v>40.200000000000003</v>
       </c>
-      <c r="J37" s="245" t="s">
+      <c r="J37" s="194" t="s">
         <v>256</v>
       </c>
       <c r="K37" s="139" t="s">
@@ -33867,26 +33875,26 @@
       </c>
     </row>
     <row r="38" spans="1:15" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A38" s="239"/>
+      <c r="A38" s="196"/>
       <c r="B38" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="241">
+      <c r="C38" s="175">
         <v>59.8</v>
       </c>
-      <c r="D38" s="241">
+      <c r="D38" s="175">
         <v>40.200000000000003</v>
       </c>
       <c r="E38" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F38" s="240">
+      <c r="F38" s="174">
         <v>81.8</v>
       </c>
-      <c r="G38" s="240">
+      <c r="G38" s="174">
         <v>18.2</v>
       </c>
-      <c r="J38" s="245"/>
+      <c r="J38" s="194"/>
       <c r="K38" s="139" t="s">
         <v>47</v>
       </c>
@@ -33898,25 +33906,25 @@
       </c>
     </row>
     <row r="39" spans="1:15" ht="15.6" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B39" s="243" t="s">
+      <c r="B39" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="C39" s="224">
+      <c r="C39" s="167">
         <v>64.099999999999994</v>
       </c>
-      <c r="D39" s="224">
+      <c r="D39" s="167">
         <v>35.9</v>
       </c>
-      <c r="E39" s="243" t="s">
+      <c r="E39" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="F39" s="224">
+      <c r="F39" s="167">
         <v>64.099999999999994</v>
       </c>
-      <c r="G39" s="224">
+      <c r="G39" s="167">
         <v>35.9</v>
       </c>
-      <c r="J39" s="245"/>
+      <c r="J39" s="194"/>
       <c r="K39" s="139" t="s">
         <v>151</v>
       </c>
@@ -33952,22 +33960,22 @@
       <c r="I45" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="J45" s="241">
+      <c r="J45" s="175">
         <v>59.1</v>
       </c>
-      <c r="K45" s="241">
+      <c r="K45" s="175">
         <v>64.900000000000006</v>
       </c>
-      <c r="L45" s="241">
+      <c r="L45" s="175">
         <v>46.9</v>
       </c>
-      <c r="M45" s="241">
+      <c r="M45" s="175">
         <v>65.3</v>
       </c>
-      <c r="N45" s="241">
+      <c r="N45" s="175">
         <v>33.6</v>
       </c>
-      <c r="O45" s="241">
+      <c r="O45" s="175">
         <v>59.8</v>
       </c>
     </row>
@@ -33975,22 +33983,22 @@
       <c r="I46" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="J46" s="240">
+      <c r="J46" s="174">
         <v>79.900000000000006</v>
       </c>
-      <c r="K46" s="240">
+      <c r="K46" s="174">
         <v>89.1</v>
       </c>
-      <c r="L46" s="240">
+      <c r="L46" s="174">
         <v>75.5</v>
       </c>
-      <c r="M46" s="240">
+      <c r="M46" s="174">
         <v>55</v>
       </c>
-      <c r="N46" s="240">
+      <c r="N46" s="174">
         <v>21</v>
       </c>
-      <c r="O46" s="240">
+      <c r="O46" s="174">
         <v>81.8</v>
       </c>
     </row>
@@ -34019,11 +34027,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="J22:J24"/>
-    <mergeCell ref="J25:J27"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="J31:J33"/>
-    <mergeCell ref="J34:J36"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
     <mergeCell ref="J37:J39"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="A22:A23"/>
@@ -34035,14 +34046,11 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="D20:D21"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="J25:J27"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="J31:J33"/>
+    <mergeCell ref="J34:J36"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -34056,79 +34064,79 @@
   <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="182" t="s">
+      <c r="A1" s="222" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="182" t="s">
+      <c r="B1" s="222" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="182" t="s">
+      <c r="C1" s="222" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="182" t="s">
+      <c r="D1" s="222" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="185" t="s">
+      <c r="E1" s="225" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
-      <c r="I1" s="186"/>
-      <c r="J1" s="186"/>
-      <c r="K1" s="186"/>
-      <c r="L1" s="187"/>
+      <c r="F1" s="226"/>
+      <c r="G1" s="226"/>
+      <c r="H1" s="226"/>
+      <c r="I1" s="226"/>
+      <c r="J1" s="226"/>
+      <c r="K1" s="226"/>
+      <c r="L1" s="227"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="183"/>
-      <c r="B2" s="183"/>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
+      <c r="A2" s="223"/>
+      <c r="B2" s="223"/>
+      <c r="C2" s="223"/>
+      <c r="D2" s="223"/>
       <c r="E2" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="178" t="s">
+      <c r="F2" s="218" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="178" t="s">
+      <c r="G2" s="218" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="178" t="s">
+      <c r="H2" s="218" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="178" t="s">
+      <c r="I2" s="218" t="s">
         <v>30</v>
       </c>
       <c r="J2" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="178" t="s">
+      <c r="K2" s="218" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="178" t="s">
+      <c r="L2" s="218" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="184"/>
-      <c r="B3" s="184"/>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
+      <c r="A3" s="224"/>
+      <c r="B3" s="224"/>
+      <c r="C3" s="224"/>
+      <c r="D3" s="224"/>
       <c r="E3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="179"/>
-      <c r="G3" s="179"/>
-      <c r="H3" s="179"/>
-      <c r="I3" s="179"/>
+      <c r="F3" s="219"/>
+      <c r="G3" s="219"/>
+      <c r="H3" s="219"/>
+      <c r="I3" s="219"/>
       <c r="J3" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="179"/>
-      <c r="L3" s="179"/>
+      <c r="K3" s="219"/>
+      <c r="L3" s="219"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="180" t="s">
+      <c r="A4" s="220" t="s">
         <v>73</v>
       </c>
       <c r="B4" s="34" t="s">
@@ -34166,7 +34174,7 @@
       </c>
     </row>
     <row r="5" spans="1:12">
-      <c r="A5" s="181"/>
+      <c r="A5" s="221"/>
       <c r="B5" s="36" t="s">
         <v>14</v>
       </c>
@@ -34202,7 +34210,7 @@
       </c>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="180" t="s">
+      <c r="A6" s="220" t="s">
         <v>74</v>
       </c>
       <c r="B6" s="34" t="s">
@@ -34240,7 +34248,7 @@
       </c>
     </row>
     <row r="7" spans="1:12">
-      <c r="A7" s="181"/>
+      <c r="A7" s="221"/>
       <c r="B7" s="36" t="s">
         <v>14</v>
       </c>
@@ -34276,7 +34284,7 @@
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="180" t="s">
+      <c r="A8" s="220" t="s">
         <v>77</v>
       </c>
       <c r="B8" s="34" t="s">
@@ -34314,7 +34322,7 @@
       </c>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="181"/>
+      <c r="A9" s="221"/>
       <c r="B9" s="36" t="s">
         <v>14</v>
       </c>
@@ -34392,8 +34400,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="18" thickTop="1" thickBot="1">
-      <c r="A2" s="189"/>
-      <c r="B2" s="190"/>
+      <c r="A2" s="264"/>
+      <c r="B2" s="265"/>
       <c r="C2" s="25" t="s">
         <v>5</v>
       </c>
@@ -34405,10 +34413,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="18" thickTop="1" thickBot="1">
-      <c r="A3" s="191" t="s">
+      <c r="A3" s="231" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="192"/>
+      <c r="B3" s="232"/>
       <c r="C3" s="58">
         <v>49.3</v>
       </c>
@@ -34424,7 +34432,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="17.25" thickTop="1">
-      <c r="A4" s="193" t="s">
+      <c r="A4" s="233" t="s">
         <v>83</v>
       </c>
       <c r="B4" s="43" t="s">
@@ -34440,12 +34448,12 @@
         <v>62.3</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F30" si="0">E4-C4</f>
+        <f t="shared" ref="F4:F28" si="0">E4-C4</f>
         <v>15.099999999999994</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="194"/>
+      <c r="A5" s="234"/>
       <c r="B5" s="19" t="s">
         <v>85</v>
       </c>
@@ -34464,7 +34472,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="195" t="s">
+      <c r="A6" s="235" t="s">
         <v>86</v>
       </c>
       <c r="B6" s="46" t="s">
@@ -34485,7 +34493,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="196"/>
+      <c r="A7" s="236"/>
       <c r="B7" s="47" t="s">
         <v>88</v>
       </c>
@@ -34504,7 +34512,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="196"/>
+      <c r="A8" s="236"/>
       <c r="B8" s="47" t="s">
         <v>89</v>
       </c>
@@ -34523,7 +34531,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="196"/>
+      <c r="A9" s="236"/>
       <c r="B9" s="47" t="s">
         <v>90</v>
       </c>
@@ -34542,7 +34550,7 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="196"/>
+      <c r="A10" s="236"/>
       <c r="B10" s="47" t="s">
         <v>91</v>
       </c>
@@ -34561,7 +34569,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="194"/>
+      <c r="A11" s="234"/>
       <c r="B11" s="49" t="s">
         <v>92</v>
       </c>
@@ -34580,7 +34588,7 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="195" t="s">
+      <c r="A12" s="235" t="s">
         <v>93</v>
       </c>
       <c r="B12" s="50" t="s">
@@ -34601,7 +34609,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="24">
-      <c r="A13" s="196"/>
+      <c r="A13" s="236"/>
       <c r="B13" s="18" t="s">
         <v>98</v>
       </c>
@@ -34620,7 +34628,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="36">
-      <c r="A14" s="196"/>
+      <c r="A14" s="236"/>
       <c r="B14" s="18" t="s">
         <v>99</v>
       </c>
@@ -34639,7 +34647,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="36">
-      <c r="A15" s="196"/>
+      <c r="A15" s="236"/>
       <c r="B15" s="18" t="s">
         <v>100</v>
       </c>
@@ -34658,7 +34666,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="24">
-      <c r="A16" s="196"/>
+      <c r="A16" s="236"/>
       <c r="B16" s="18" t="s">
         <v>101</v>
       </c>
@@ -34677,7 +34685,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="36">
-      <c r="A17" s="196"/>
+      <c r="A17" s="236"/>
       <c r="B17" s="18" t="s">
         <v>102</v>
       </c>
@@ -34696,7 +34704,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="24">
-      <c r="A18" s="194"/>
+      <c r="A18" s="234"/>
       <c r="B18" s="19" t="s">
         <v>103</v>
       </c>
@@ -34898,13 +34906,13 @@
       <c r="B28" s="18" t="s">
         <v>262</v>
       </c>
-      <c r="C28" s="247">
+      <c r="C28" s="179">
         <v>13</v>
       </c>
-      <c r="D28" s="271">
+      <c r="D28" s="193">
         <v>43.8</v>
       </c>
-      <c r="E28" s="248">
+      <c r="E28" s="180">
         <v>39</v>
       </c>
       <c r="F28">
@@ -34921,13 +34929,13 @@
       <c r="F29" s="57"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="C30" s="247"/>
-      <c r="D30" s="271"/>
-      <c r="E30" s="248"/>
+      <c r="C30" s="179"/>
+      <c r="D30" s="193"/>
+      <c r="E30" s="180"/>
     </row>
     <row r="67" spans="3:13" ht="24">
-      <c r="C67" s="188"/>
-      <c r="D67" s="188"/>
+      <c r="C67" s="263"/>
+      <c r="D67" s="263"/>
       <c r="E67" s="72" t="s">
         <v>107</v>
       </c>
@@ -34950,10 +34958,10 @@
       </c>
     </row>
     <row r="68" spans="3:13">
-      <c r="C68" s="215" t="s">
+      <c r="C68" s="257" t="s">
         <v>82</v>
       </c>
-      <c r="D68" s="215"/>
+      <c r="D68" s="257"/>
       <c r="E68" s="73">
         <v>49.3</v>
       </c>
@@ -34964,7 +34972,7 @@
         <v>12.900000000000006</v>
       </c>
       <c r="H68" s="56"/>
-      <c r="I68" s="205" t="s">
+      <c r="I68" s="246" t="s">
         <v>83</v>
       </c>
       <c r="J68" s="72" t="s">
@@ -34982,7 +34990,7 @@
       </c>
     </row>
     <row r="69" spans="3:13">
-      <c r="C69" s="205" t="s">
+      <c r="C69" s="246" t="s">
         <v>83</v>
       </c>
       <c r="D69" s="72" t="s">
@@ -34998,7 +35006,7 @@
         <v>15.099999999999994</v>
       </c>
       <c r="H69" s="56"/>
-      <c r="I69" s="205"/>
+      <c r="I69" s="246"/>
       <c r="J69" s="72" t="s">
         <v>144</v>
       </c>
@@ -35014,7 +35022,7 @@
       </c>
     </row>
     <row r="70" spans="3:13">
-      <c r="C70" s="205"/>
+      <c r="C70" s="246"/>
       <c r="D70" s="72" t="s">
         <v>85</v>
       </c>
@@ -35028,7 +35036,7 @@
         <v>10.900000000000006</v>
       </c>
       <c r="H70" s="56"/>
-      <c r="I70" s="208" t="s">
+      <c r="I70" s="247" t="s">
         <v>138</v>
       </c>
       <c r="J70" s="72" t="s">
@@ -35046,7 +35054,7 @@
       </c>
     </row>
     <row r="71" spans="3:13">
-      <c r="C71" s="205" t="s">
+      <c r="C71" s="246" t="s">
         <v>86</v>
       </c>
       <c r="D71" s="77" t="s">
@@ -35062,7 +35070,7 @@
         <v>6.2999999999999972</v>
       </c>
       <c r="H71" s="56"/>
-      <c r="I71" s="209"/>
+      <c r="I71" s="248"/>
       <c r="J71" s="72" t="s">
         <v>128</v>
       </c>
@@ -35078,7 +35086,7 @@
       </c>
     </row>
     <row r="72" spans="3:13">
-      <c r="C72" s="205"/>
+      <c r="C72" s="246"/>
       <c r="D72" s="77" t="s">
         <v>88</v>
       </c>
@@ -35092,7 +35100,7 @@
         <v>19.200000000000003</v>
       </c>
       <c r="H72" s="56"/>
-      <c r="I72" s="209"/>
+      <c r="I72" s="248"/>
       <c r="J72" s="72" t="s">
         <v>129</v>
       </c>
@@ -35108,7 +35116,7 @@
       </c>
     </row>
     <row r="73" spans="3:13">
-      <c r="C73" s="205"/>
+      <c r="C73" s="246"/>
       <c r="D73" s="77" t="s">
         <v>89</v>
       </c>
@@ -35122,7 +35130,7 @@
         <v>12.899999999999991</v>
       </c>
       <c r="H73" s="56"/>
-      <c r="I73" s="209"/>
+      <c r="I73" s="248"/>
       <c r="J73" s="72" t="s">
         <v>130</v>
       </c>
@@ -35138,7 +35146,7 @@
       </c>
     </row>
     <row r="74" spans="3:13">
-      <c r="C74" s="205"/>
+      <c r="C74" s="246"/>
       <c r="D74" s="77" t="s">
         <v>90</v>
       </c>
@@ -35152,7 +35160,7 @@
         <v>10.100000000000009</v>
       </c>
       <c r="H74" s="56"/>
-      <c r="I74" s="209"/>
+      <c r="I74" s="248"/>
       <c r="J74" s="72" t="s">
         <v>131</v>
       </c>
@@ -35168,7 +35176,7 @@
       </c>
     </row>
     <row r="75" spans="3:13">
-      <c r="C75" s="205"/>
+      <c r="C75" s="246"/>
       <c r="D75" s="77" t="s">
         <v>91</v>
       </c>
@@ -35182,7 +35190,7 @@
         <v>13.199999999999996</v>
       </c>
       <c r="H75" s="56"/>
-      <c r="I75" s="210"/>
+      <c r="I75" s="249"/>
       <c r="J75" s="72" t="s">
         <v>132</v>
       </c>
@@ -35198,7 +35206,7 @@
       </c>
     </row>
     <row r="76" spans="3:13">
-      <c r="C76" s="205"/>
+      <c r="C76" s="246"/>
       <c r="D76" s="77" t="s">
         <v>92</v>
       </c>
@@ -35212,7 +35220,7 @@
         <v>16.899999999999999</v>
       </c>
       <c r="H76" s="56"/>
-      <c r="I76" s="208" t="s">
+      <c r="I76" s="247" t="s">
         <v>139</v>
       </c>
       <c r="J76" s="72" t="s">
@@ -35230,7 +35238,7 @@
       </c>
     </row>
     <row r="77" spans="3:13">
-      <c r="C77" s="205" t="s">
+      <c r="C77" s="246" t="s">
         <v>139</v>
       </c>
       <c r="D77" s="72" t="s">
@@ -35246,7 +35254,7 @@
         <v>13.399999999999999</v>
       </c>
       <c r="H77" s="56"/>
-      <c r="I77" s="209"/>
+      <c r="I77" s="248"/>
       <c r="J77" s="72" t="s">
         <v>113</v>
       </c>
@@ -35262,7 +35270,7 @@
       </c>
     </row>
     <row r="78" spans="3:13" ht="16.5" customHeight="1">
-      <c r="C78" s="205"/>
+      <c r="C78" s="246"/>
       <c r="D78" s="72" t="s">
         <v>114</v>
       </c>
@@ -35276,7 +35284,7 @@
         <v>12.899999999999991</v>
       </c>
       <c r="H78" s="56"/>
-      <c r="I78" s="209"/>
+      <c r="I78" s="248"/>
       <c r="J78" s="72" t="s">
         <v>133</v>
       </c>
@@ -35292,7 +35300,7 @@
       </c>
     </row>
     <row r="79" spans="3:13" ht="16.5" customHeight="1">
-      <c r="C79" s="205"/>
+      <c r="C79" s="246"/>
       <c r="D79" s="72" t="s">
         <v>115</v>
       </c>
@@ -35306,7 +35314,7 @@
         <v>8.3000000000000043</v>
       </c>
       <c r="H79" s="56"/>
-      <c r="I79" s="209"/>
+      <c r="I79" s="248"/>
       <c r="J79" s="72" t="s">
         <v>116</v>
       </c>
@@ -35322,7 +35330,7 @@
       </c>
     </row>
     <row r="80" spans="3:13">
-      <c r="C80" s="205"/>
+      <c r="C80" s="246"/>
       <c r="D80" s="72" t="s">
         <v>117</v>
       </c>
@@ -35336,7 +35344,7 @@
         <v>10.399999999999991</v>
       </c>
       <c r="H80" s="56"/>
-      <c r="I80" s="209"/>
+      <c r="I80" s="248"/>
       <c r="J80" s="72" t="s">
         <v>118</v>
       </c>
@@ -35352,7 +35360,7 @@
       </c>
     </row>
     <row r="81" spans="3:13" ht="16.5" customHeight="1">
-      <c r="C81" s="205"/>
+      <c r="C81" s="246"/>
       <c r="D81" s="72" t="s">
         <v>119</v>
       </c>
@@ -35366,7 +35374,7 @@
         <v>13.600000000000001</v>
       </c>
       <c r="H81" s="56"/>
-      <c r="I81" s="209"/>
+      <c r="I81" s="248"/>
       <c r="J81" s="72" t="s">
         <v>120</v>
       </c>
@@ -35382,7 +35390,7 @@
       </c>
     </row>
     <row r="82" spans="3:13">
-      <c r="C82" s="205"/>
+      <c r="C82" s="246"/>
       <c r="D82" s="72" t="s">
         <v>121</v>
       </c>
@@ -35396,7 +35404,7 @@
         <v>17.100000000000001</v>
       </c>
       <c r="H82" s="56"/>
-      <c r="I82" s="210"/>
+      <c r="I82" s="249"/>
       <c r="J82" s="72" t="s">
         <v>122</v>
       </c>
@@ -35412,7 +35420,7 @@
       </c>
     </row>
     <row r="83" spans="3:13">
-      <c r="C83" s="205"/>
+      <c r="C83" s="246"/>
       <c r="D83" s="72" t="s">
         <v>123</v>
       </c>
@@ -35426,7 +35434,7 @@
         <v>12.399999999999999</v>
       </c>
       <c r="H83" s="56"/>
-      <c r="I83" s="205" t="s">
+      <c r="I83" s="246" t="s">
         <v>111</v>
       </c>
       <c r="J83" s="72" t="s">
@@ -35444,7 +35452,7 @@
       </c>
     </row>
     <row r="84" spans="3:13">
-      <c r="C84" s="205" t="s">
+      <c r="C84" s="246" t="s">
         <v>111</v>
       </c>
       <c r="D84" s="72" t="s">
@@ -35460,7 +35468,7 @@
         <v>4.6000000000000085</v>
       </c>
       <c r="H84" s="56"/>
-      <c r="I84" s="205"/>
+      <c r="I84" s="246"/>
       <c r="J84" s="72" t="s">
         <v>35</v>
       </c>
@@ -35476,7 +35484,7 @@
       </c>
     </row>
     <row r="85" spans="3:13">
-      <c r="C85" s="205"/>
+      <c r="C85" s="246"/>
       <c r="D85" s="72" t="s">
         <v>35</v>
       </c>
@@ -35490,7 +35498,7 @@
         <v>15.299999999999997</v>
       </c>
       <c r="H85" s="56"/>
-      <c r="I85" s="205"/>
+      <c r="I85" s="246"/>
       <c r="J85" s="72" t="s">
         <v>36</v>
       </c>
@@ -35506,7 +35514,7 @@
       </c>
     </row>
     <row r="86" spans="3:13">
-      <c r="C86" s="205"/>
+      <c r="C86" s="246"/>
       <c r="D86" s="72" t="s">
         <v>36</v>
       </c>
@@ -35523,7 +35531,7 @@
       <c r="J86" s="72"/>
     </row>
     <row r="87" spans="3:13">
-      <c r="C87" s="205" t="s">
+      <c r="C87" s="246" t="s">
         <v>112</v>
       </c>
       <c r="D87" s="72" t="s">
@@ -35541,7 +35549,7 @@
       <c r="H87" s="56"/>
     </row>
     <row r="88" spans="3:13">
-      <c r="C88" s="205"/>
+      <c r="C88" s="246"/>
       <c r="D88" s="72" t="s">
         <v>27</v>
       </c>
@@ -35557,7 +35565,7 @@
       <c r="H88" s="56"/>
     </row>
     <row r="89" spans="3:13">
-      <c r="C89" s="205"/>
+      <c r="C89" s="246"/>
       <c r="D89" s="72" t="s">
         <v>28</v>
       </c>
@@ -35573,7 +35581,7 @@
       <c r="H89" s="56"/>
     </row>
     <row r="90" spans="3:13">
-      <c r="C90" s="205"/>
+      <c r="C90" s="246"/>
       <c r="D90" s="72" t="s">
         <v>30</v>
       </c>
@@ -35589,7 +35597,7 @@
       <c r="H90" s="56"/>
     </row>
     <row r="91" spans="3:13">
-      <c r="C91" s="205"/>
+      <c r="C91" s="246"/>
       <c r="D91" s="72" t="s">
         <v>29</v>
       </c>
@@ -35605,7 +35613,7 @@
       <c r="H91" s="56"/>
     </row>
     <row r="92" spans="3:13">
-      <c r="C92" s="205"/>
+      <c r="C92" s="246"/>
       <c r="D92" s="72" t="s">
         <v>105</v>
       </c>
@@ -35621,7 +35629,7 @@
       <c r="H92" s="56"/>
     </row>
     <row r="93" spans="3:13">
-      <c r="C93" s="205"/>
+      <c r="C93" s="246"/>
       <c r="D93" s="72" t="s">
         <v>106</v>
       </c>
@@ -35637,7 +35645,7 @@
       <c r="H93" s="56"/>
     </row>
     <row r="94" spans="3:13">
-      <c r="C94" s="205"/>
+      <c r="C94" s="246"/>
       <c r="D94" s="72" t="s">
         <v>55</v>
       </c>
@@ -35654,40 +35662,40 @@
     </row>
     <row r="101" spans="2:21" ht="17.25" thickBot="1"/>
     <row r="102" spans="2:21" ht="17.25" thickBot="1">
-      <c r="B102" s="211" t="s">
+      <c r="B102" s="250" t="s">
         <v>124</v>
       </c>
-      <c r="C102" s="212"/>
-      <c r="D102" s="204" t="s">
+      <c r="C102" s="251"/>
+      <c r="D102" s="262" t="s">
         <v>83</v>
       </c>
-      <c r="E102" s="199"/>
-      <c r="F102" s="197" t="s">
+      <c r="E102" s="256"/>
+      <c r="F102" s="254" t="s">
         <v>138</v>
       </c>
-      <c r="G102" s="198"/>
-      <c r="H102" s="198"/>
-      <c r="I102" s="198"/>
-      <c r="J102" s="198"/>
-      <c r="K102" s="199"/>
-      <c r="L102" s="197" t="s">
+      <c r="G102" s="255"/>
+      <c r="H102" s="255"/>
+      <c r="I102" s="255"/>
+      <c r="J102" s="255"/>
+      <c r="K102" s="256"/>
+      <c r="L102" s="254" t="s">
         <v>139</v>
       </c>
-      <c r="M102" s="198"/>
-      <c r="N102" s="198"/>
-      <c r="O102" s="198"/>
-      <c r="P102" s="198"/>
-      <c r="Q102" s="198"/>
-      <c r="R102" s="199"/>
-      <c r="S102" s="200" t="s">
+      <c r="M102" s="255"/>
+      <c r="N102" s="255"/>
+      <c r="O102" s="255"/>
+      <c r="P102" s="255"/>
+      <c r="Q102" s="255"/>
+      <c r="R102" s="256"/>
+      <c r="S102" s="258" t="s">
         <v>140</v>
       </c>
-      <c r="T102" s="198"/>
-      <c r="U102" s="201"/>
+      <c r="T102" s="255"/>
+      <c r="U102" s="259"/>
     </row>
     <row r="103" spans="2:21" ht="23.25" thickBot="1">
-      <c r="B103" s="213"/>
-      <c r="C103" s="214"/>
+      <c r="B103" s="252"/>
+      <c r="C103" s="253"/>
       <c r="D103" s="78" t="s">
         <v>125</v>
       </c>
@@ -35806,7 +35814,7 @@
       </c>
     </row>
     <row r="105" spans="2:21" ht="23.25" thickBot="1">
-      <c r="B105" s="202" t="s">
+      <c r="B105" s="260" t="s">
         <v>135</v>
       </c>
       <c r="C105" s="84" t="s">
@@ -35868,7 +35876,7 @@
       </c>
     </row>
     <row r="106" spans="2:21" ht="23.25" thickBot="1">
-      <c r="B106" s="203"/>
+      <c r="B106" s="261"/>
       <c r="C106" s="87" t="s">
         <v>137</v>
       </c>
@@ -36012,7 +36020,7 @@
       </c>
     </row>
     <row r="110" spans="2:21">
-      <c r="C110" s="206" t="s">
+      <c r="C110" s="244" t="s">
         <v>83</v>
       </c>
       <c r="D110" s="91" t="s">
@@ -36030,7 +36038,7 @@
       </c>
     </row>
     <row r="111" spans="2:21">
-      <c r="C111" s="206"/>
+      <c r="C111" s="244"/>
       <c r="D111" s="91" t="s">
         <v>126</v>
       </c>
@@ -36046,7 +36054,7 @@
       </c>
     </row>
     <row r="112" spans="2:21">
-      <c r="C112" s="207" t="s">
+      <c r="C112" s="245" t="s">
         <v>138</v>
       </c>
       <c r="D112" s="91" t="s">
@@ -36064,7 +36072,7 @@
       </c>
     </row>
     <row r="113" spans="3:7">
-      <c r="C113" s="206"/>
+      <c r="C113" s="244"/>
       <c r="D113" s="91" t="s">
         <v>128</v>
       </c>
@@ -36080,7 +36088,7 @@
       </c>
     </row>
     <row r="114" spans="3:7">
-      <c r="C114" s="206"/>
+      <c r="C114" s="244"/>
       <c r="D114" s="91" t="s">
         <v>129</v>
       </c>
@@ -36096,7 +36104,7 @@
       </c>
     </row>
     <row r="115" spans="3:7">
-      <c r="C115" s="206"/>
+      <c r="C115" s="244"/>
       <c r="D115" s="91" t="s">
         <v>130</v>
       </c>
@@ -36112,7 +36120,7 @@
       </c>
     </row>
     <row r="116" spans="3:7">
-      <c r="C116" s="206"/>
+      <c r="C116" s="244"/>
       <c r="D116" s="91" t="s">
         <v>131</v>
       </c>
@@ -36128,7 +36136,7 @@
       </c>
     </row>
     <row r="117" spans="3:7">
-      <c r="C117" s="206"/>
+      <c r="C117" s="244"/>
       <c r="D117" s="91" t="s">
         <v>132</v>
       </c>
@@ -36144,7 +36152,7 @@
       </c>
     </row>
     <row r="118" spans="3:7">
-      <c r="C118" s="207" t="s">
+      <c r="C118" s="245" t="s">
         <v>139</v>
       </c>
       <c r="D118" s="91" t="s">
@@ -36162,7 +36170,7 @@
       </c>
     </row>
     <row r="119" spans="3:7">
-      <c r="C119" s="206"/>
+      <c r="C119" s="244"/>
       <c r="D119" s="91" t="s">
         <v>113</v>
       </c>
@@ -36178,7 +36186,7 @@
       </c>
     </row>
     <row r="120" spans="3:7" ht="22.5">
-      <c r="C120" s="206"/>
+      <c r="C120" s="244"/>
       <c r="D120" s="91" t="s">
         <v>133</v>
       </c>
@@ -36194,7 +36202,7 @@
       </c>
     </row>
     <row r="121" spans="3:7" ht="22.5">
-      <c r="C121" s="206"/>
+      <c r="C121" s="244"/>
       <c r="D121" s="91" t="s">
         <v>116</v>
       </c>
@@ -36210,7 +36218,7 @@
       </c>
     </row>
     <row r="122" spans="3:7">
-      <c r="C122" s="206"/>
+      <c r="C122" s="244"/>
       <c r="D122" s="91" t="s">
         <v>118</v>
       </c>
@@ -36226,7 +36234,7 @@
       </c>
     </row>
     <row r="123" spans="3:7" ht="22.5">
-      <c r="C123" s="206"/>
+      <c r="C123" s="244"/>
       <c r="D123" s="91" t="s">
         <v>120</v>
       </c>
@@ -36242,7 +36250,7 @@
       </c>
     </row>
     <row r="124" spans="3:7">
-      <c r="C124" s="206"/>
+      <c r="C124" s="244"/>
       <c r="D124" s="91" t="s">
         <v>122</v>
       </c>
@@ -36258,7 +36266,7 @@
       </c>
     </row>
     <row r="125" spans="3:7">
-      <c r="C125" s="207" t="s">
+      <c r="C125" s="245" t="s">
         <v>140</v>
       </c>
       <c r="D125" s="91" t="s">
@@ -36276,7 +36284,7 @@
       </c>
     </row>
     <row r="126" spans="3:7">
-      <c r="C126" s="206"/>
+      <c r="C126" s="244"/>
       <c r="D126" s="91" t="s">
         <v>35</v>
       </c>
@@ -36292,7 +36300,7 @@
       </c>
     </row>
     <row r="127" spans="3:7">
-      <c r="C127" s="206"/>
+      <c r="C127" s="244"/>
       <c r="D127" s="91" t="s">
         <v>36</v>
       </c>
@@ -36309,9 +36317,9 @@
     </row>
     <row r="138" spans="2:13" ht="17.25" thickBot="1"/>
     <row r="139" spans="2:13" ht="17.25" thickTop="1">
-      <c r="B139" s="261"/>
-      <c r="C139" s="226"/>
-      <c r="D139" s="228" t="s">
+      <c r="B139" s="237"/>
+      <c r="C139" s="197"/>
+      <c r="D139" s="203" t="s">
         <v>245</v>
       </c>
       <c r="E139" s="16" t="s">
@@ -36329,23 +36337,23 @@
       <c r="I139" s="16" t="s">
         <v>269</v>
       </c>
-      <c r="J139" s="230" t="s">
+      <c r="J139" s="199" t="s">
         <v>168</v>
       </c>
-      <c r="K139" s="230" t="s">
+      <c r="K139" s="199" t="s">
         <v>81</v>
       </c>
-      <c r="L139" s="232" t="s">
+      <c r="L139" s="201" t="s">
         <v>249</v>
       </c>
-      <c r="M139" s="268" t="s">
+      <c r="M139" s="228" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="140" spans="2:13">
-      <c r="B140" s="262"/>
-      <c r="C140" s="263"/>
-      <c r="D140" s="265"/>
+      <c r="B140" s="238"/>
+      <c r="C140" s="239"/>
+      <c r="D140" s="241"/>
       <c r="E140" s="114" t="s">
         <v>263</v>
       </c>
@@ -36361,105 +36369,105 @@
       <c r="I140" s="114" t="s">
         <v>270</v>
       </c>
-      <c r="J140" s="266"/>
-      <c r="K140" s="266"/>
-      <c r="L140" s="267"/>
-      <c r="M140" s="269"/>
+      <c r="J140" s="242"/>
+      <c r="K140" s="242"/>
+      <c r="L140" s="243"/>
+      <c r="M140" s="229"/>
     </row>
     <row r="141" spans="2:13" ht="17.25" thickBot="1">
-      <c r="B141" s="264"/>
-      <c r="C141" s="227"/>
-      <c r="D141" s="229"/>
-      <c r="E141" s="222" t="s">
+      <c r="B141" s="240"/>
+      <c r="C141" s="198"/>
+      <c r="D141" s="204"/>
+      <c r="E141" s="165" t="s">
         <v>264</v>
       </c>
-      <c r="F141" s="249"/>
-      <c r="G141" s="249"/>
-      <c r="H141" s="222" t="s">
+      <c r="F141" s="181"/>
+      <c r="G141" s="181"/>
+      <c r="H141" s="165" t="s">
         <v>264</v>
       </c>
-      <c r="I141" s="249"/>
-      <c r="J141" s="231"/>
-      <c r="K141" s="231"/>
-      <c r="L141" s="233"/>
-      <c r="M141" s="270"/>
+      <c r="I141" s="181"/>
+      <c r="J141" s="200"/>
+      <c r="K141" s="200"/>
+      <c r="L141" s="202"/>
+      <c r="M141" s="230"/>
     </row>
     <row r="142" spans="2:13" ht="18" thickTop="1" thickBot="1">
-      <c r="B142" s="191" t="s">
+      <c r="B142" s="231" t="s">
         <v>82</v>
       </c>
-      <c r="C142" s="192"/>
-      <c r="D142" s="223">
+      <c r="C142" s="232"/>
+      <c r="D142" s="166">
         <v>-2207</v>
       </c>
-      <c r="E142" s="223">
+      <c r="E142" s="166">
         <v>18.100000000000001</v>
       </c>
-      <c r="F142" s="223">
+      <c r="F142" s="166">
         <v>13.6</v>
       </c>
-      <c r="G142" s="223">
+      <c r="G142" s="166">
         <v>26.4</v>
       </c>
-      <c r="H142" s="223">
+      <c r="H142" s="166">
         <v>36.299999999999997</v>
       </c>
-      <c r="I142" s="223">
+      <c r="I142" s="166">
         <v>5.6</v>
       </c>
-      <c r="J142" s="224">
+      <c r="J142" s="167">
         <v>31.7</v>
       </c>
-      <c r="K142" s="224">
+      <c r="K142" s="167">
         <v>62.7</v>
       </c>
-      <c r="L142" s="225">
+      <c r="L142" s="168">
         <v>2.9</v>
       </c>
-      <c r="M142" s="250">
+      <c r="M142" s="182">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="143" spans="2:13" ht="17.25" thickTop="1">
-      <c r="B143" s="193" t="s">
+      <c r="B143" s="233" t="s">
         <v>83</v>
       </c>
       <c r="C143" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="D143" s="251">
+      <c r="D143" s="183">
         <v>-1094</v>
       </c>
-      <c r="E143" s="251">
+      <c r="E143" s="183">
         <v>18.2</v>
       </c>
-      <c r="F143" s="251">
+      <c r="F143" s="183">
         <v>14.9</v>
       </c>
-      <c r="G143" s="251">
+      <c r="G143" s="183">
         <v>25.5</v>
       </c>
-      <c r="H143" s="251">
+      <c r="H143" s="183">
         <v>37</v>
       </c>
-      <c r="I143" s="251">
+      <c r="I143" s="183">
         <v>4.4000000000000004</v>
       </c>
-      <c r="J143" s="252">
+      <c r="J143" s="184">
         <v>33.1</v>
       </c>
-      <c r="K143" s="252">
+      <c r="K143" s="184">
         <v>62.5</v>
       </c>
-      <c r="L143" s="253">
+      <c r="L143" s="185">
         <v>2.9</v>
       </c>
-      <c r="M143" s="254">
+      <c r="M143" s="186">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="144" spans="2:13">
-      <c r="B144" s="194"/>
+      <c r="B144" s="234"/>
       <c r="C144" s="19" t="s">
         <v>85</v>
       </c>
@@ -36481,59 +36489,59 @@
       <c r="I144" s="44">
         <v>6.8</v>
       </c>
-      <c r="J144" s="236">
+      <c r="J144" s="171">
         <v>30.4</v>
       </c>
-      <c r="K144" s="236">
+      <c r="K144" s="171">
         <v>62.8</v>
       </c>
-      <c r="L144" s="237">
+      <c r="L144" s="172">
         <v>2.9</v>
       </c>
-      <c r="M144" s="255">
+      <c r="M144" s="187">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="145" spans="2:13">
-      <c r="B145" s="195" t="s">
+      <c r="B145" s="235" t="s">
         <v>86</v>
       </c>
       <c r="C145" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="D145" s="256">
+      <c r="D145" s="188">
         <v>-333</v>
       </c>
-      <c r="E145" s="256">
+      <c r="E145" s="188">
         <v>19.2</v>
       </c>
-      <c r="F145" s="256">
+      <c r="F145" s="188">
         <v>17.600000000000001</v>
       </c>
-      <c r="G145" s="256">
+      <c r="G145" s="188">
         <v>33.799999999999997</v>
       </c>
-      <c r="H145" s="256">
+      <c r="H145" s="188">
         <v>22.2</v>
       </c>
-      <c r="I145" s="256">
+      <c r="I145" s="188">
         <v>7.2</v>
       </c>
-      <c r="J145" s="257">
+      <c r="J145" s="189">
         <v>36.799999999999997</v>
       </c>
-      <c r="K145" s="257">
+      <c r="K145" s="189">
         <v>56.1</v>
       </c>
-      <c r="L145" s="258">
+      <c r="L145" s="190">
         <v>2.6</v>
       </c>
-      <c r="M145" s="259">
+      <c r="M145" s="191">
         <v>1.06</v>
       </c>
     </row>
     <row r="146" spans="2:13">
-      <c r="B146" s="196"/>
+      <c r="B146" s="236"/>
       <c r="C146" s="47" t="s">
         <v>88</v>
       </c>
@@ -36555,21 +36563,21 @@
       <c r="I146" s="48">
         <v>7.1</v>
       </c>
-      <c r="J146" s="234">
+      <c r="J146" s="169">
         <v>27.4</v>
       </c>
-      <c r="K146" s="234">
+      <c r="K146" s="169">
         <v>65.5</v>
       </c>
-      <c r="L146" s="235">
+      <c r="L146" s="170">
         <v>2.9</v>
       </c>
-      <c r="M146" s="260">
+      <c r="M146" s="192">
         <v>1.05</v>
       </c>
     </row>
     <row r="147" spans="2:13">
-      <c r="B147" s="196"/>
+      <c r="B147" s="236"/>
       <c r="C147" s="47" t="s">
         <v>89</v>
       </c>
@@ -36591,21 +36599,21 @@
       <c r="I147" s="48">
         <v>3.7</v>
       </c>
-      <c r="J147" s="234">
+      <c r="J147" s="169">
         <v>17.600000000000001</v>
       </c>
-      <c r="K147" s="234">
+      <c r="K147" s="169">
         <v>78.7</v>
       </c>
-      <c r="L147" s="235">
+      <c r="L147" s="170">
         <v>3.2</v>
       </c>
-      <c r="M147" s="260">
+      <c r="M147" s="192">
         <v>1</v>
       </c>
     </row>
     <row r="148" spans="2:13">
-      <c r="B148" s="196"/>
+      <c r="B148" s="236"/>
       <c r="C148" s="47" t="s">
         <v>90</v>
       </c>
@@ -36627,21 +36635,21 @@
       <c r="I148" s="48">
         <v>2.8</v>
       </c>
-      <c r="J148" s="234">
+      <c r="J148" s="169">
         <v>24.6</v>
       </c>
-      <c r="K148" s="234">
+      <c r="K148" s="169">
         <v>72.599999999999994</v>
       </c>
-      <c r="L148" s="235">
+      <c r="L148" s="170">
         <v>3.1</v>
       </c>
-      <c r="M148" s="260">
+      <c r="M148" s="192">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="149" spans="2:13">
-      <c r="B149" s="196"/>
+      <c r="B149" s="236"/>
       <c r="C149" s="47" t="s">
         <v>91</v>
       </c>
@@ -36663,21 +36671,21 @@
       <c r="I149" s="48">
         <v>4.7</v>
       </c>
-      <c r="J149" s="234">
+      <c r="J149" s="169">
         <v>41.4</v>
       </c>
-      <c r="K149" s="234">
+      <c r="K149" s="169">
         <v>53.9</v>
       </c>
-      <c r="L149" s="235">
+      <c r="L149" s="170">
         <v>2.7</v>
       </c>
-      <c r="M149" s="260">
+      <c r="M149" s="192">
         <v>1.22</v>
       </c>
     </row>
     <row r="150" spans="2:13">
-      <c r="B150" s="194"/>
+      <c r="B150" s="234"/>
       <c r="C150" s="49" t="s">
         <v>92</v>
       </c>
@@ -36699,59 +36707,59 @@
       <c r="I150" s="44">
         <v>9.1</v>
       </c>
-      <c r="J150" s="236">
+      <c r="J150" s="171">
         <v>44.6</v>
       </c>
-      <c r="K150" s="236">
+      <c r="K150" s="171">
         <v>46.3</v>
       </c>
-      <c r="L150" s="237">
+      <c r="L150" s="172">
         <v>2.5</v>
       </c>
-      <c r="M150" s="255">
+      <c r="M150" s="187">
         <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="151" spans="2:13">
-      <c r="B151" s="195" t="s">
+      <c r="B151" s="235" t="s">
         <v>93</v>
       </c>
       <c r="C151" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="D151" s="256">
+      <c r="D151" s="188">
         <v>-412</v>
       </c>
-      <c r="E151" s="256">
+      <c r="E151" s="188">
         <v>18.3</v>
       </c>
-      <c r="F151" s="256">
+      <c r="F151" s="188">
         <v>13.7</v>
       </c>
-      <c r="G151" s="256">
+      <c r="G151" s="188">
         <v>26.3</v>
       </c>
-      <c r="H151" s="256">
+      <c r="H151" s="188">
         <v>35.4</v>
       </c>
-      <c r="I151" s="256">
+      <c r="I151" s="188">
         <v>6.2</v>
       </c>
-      <c r="J151" s="257">
+      <c r="J151" s="189">
         <v>32</v>
       </c>
-      <c r="K151" s="257">
+      <c r="K151" s="189">
         <v>61.8</v>
       </c>
-      <c r="L151" s="258">
+      <c r="L151" s="190">
         <v>2.8</v>
       </c>
-      <c r="M151" s="259">
+      <c r="M151" s="191">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="152" spans="2:13">
-      <c r="B152" s="196"/>
+      <c r="B152" s="236"/>
       <c r="C152" s="18" t="s">
         <v>271</v>
       </c>
@@ -36773,21 +36781,21 @@
       <c r="I152" s="48">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J152" s="234">
+      <c r="J152" s="169">
         <v>29.9</v>
       </c>
-      <c r="K152" s="234">
+      <c r="K152" s="169">
         <v>65.2</v>
       </c>
-      <c r="L152" s="235">
+      <c r="L152" s="170">
         <v>2.9</v>
       </c>
-      <c r="M152" s="260">
+      <c r="M152" s="192">
         <v>1.1299999999999999</v>
       </c>
     </row>
     <row r="153" spans="2:13" ht="24">
-      <c r="B153" s="196"/>
+      <c r="B153" s="236"/>
       <c r="C153" s="18" t="s">
         <v>272</v>
       </c>
@@ -36809,21 +36817,21 @@
       <c r="I153" s="48">
         <v>4.8</v>
       </c>
-      <c r="J153" s="234">
+      <c r="J153" s="169">
         <v>41.8</v>
       </c>
-      <c r="K153" s="234">
+      <c r="K153" s="169">
         <v>53.4</v>
       </c>
-      <c r="L153" s="235">
+      <c r="L153" s="170">
         <v>2.6</v>
       </c>
-      <c r="M153" s="260">
+      <c r="M153" s="192">
         <v>1.19</v>
       </c>
     </row>
     <row r="154" spans="2:13" ht="24">
-      <c r="B154" s="196"/>
+      <c r="B154" s="236"/>
       <c r="C154" s="18" t="s">
         <v>273</v>
       </c>
@@ -36845,21 +36853,21 @@
       <c r="I154" s="48">
         <v>6.5</v>
       </c>
-      <c r="J154" s="234">
+      <c r="J154" s="169">
         <v>14.9</v>
       </c>
-      <c r="K154" s="234">
+      <c r="K154" s="169">
         <v>78.599999999999994</v>
       </c>
-      <c r="L154" s="235">
+      <c r="L154" s="170">
         <v>3.3</v>
       </c>
-      <c r="M154" s="260">
+      <c r="M154" s="192">
         <v>1.01</v>
       </c>
     </row>
     <row r="155" spans="2:13">
-      <c r="B155" s="196"/>
+      <c r="B155" s="236"/>
       <c r="C155" s="18" t="s">
         <v>274</v>
       </c>
@@ -36881,21 +36889,21 @@
       <c r="I155" s="48">
         <v>5</v>
       </c>
-      <c r="J155" s="234">
+      <c r="J155" s="169">
         <v>42.2</v>
       </c>
-      <c r="K155" s="234">
+      <c r="K155" s="169">
         <v>52.9</v>
       </c>
-      <c r="L155" s="235">
+      <c r="L155" s="170">
         <v>2.6</v>
       </c>
-      <c r="M155" s="260">
+      <c r="M155" s="192">
         <v>1.0900000000000001</v>
       </c>
     </row>
     <row r="156" spans="2:13" ht="24">
-      <c r="B156" s="196"/>
+      <c r="B156" s="236"/>
       <c r="C156" s="18" t="s">
         <v>275</v>
       </c>
@@ -36917,21 +36925,21 @@
       <c r="I156" s="48">
         <v>7.4</v>
       </c>
-      <c r="J156" s="234">
+      <c r="J156" s="169">
         <v>34.6</v>
       </c>
-      <c r="K156" s="234">
+      <c r="K156" s="169">
         <v>58.1</v>
       </c>
-      <c r="L156" s="235">
+      <c r="L156" s="170">
         <v>2.8</v>
       </c>
-      <c r="M156" s="260">
+      <c r="M156" s="192">
         <v>1.1100000000000001</v>
       </c>
     </row>
     <row r="157" spans="2:13">
-      <c r="B157" s="194"/>
+      <c r="B157" s="234"/>
       <c r="C157" s="19" t="s">
         <v>276</v>
       </c>
@@ -36953,16 +36961,16 @@
       <c r="I157" s="44">
         <v>3.3</v>
       </c>
-      <c r="J157" s="236">
+      <c r="J157" s="171">
         <v>23.3</v>
       </c>
-      <c r="K157" s="236">
+      <c r="K157" s="171">
         <v>73.400000000000006</v>
       </c>
-      <c r="L157" s="237">
+      <c r="L157" s="172">
         <v>3.1</v>
       </c>
-      <c r="M157" s="255">
+      <c r="M157" s="187">
         <v>1.01</v>
       </c>
     </row>
@@ -36973,34 +36981,34 @@
       <c r="C158" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="D158" s="256">
+      <c r="D158" s="188">
         <v>-594</v>
       </c>
-      <c r="E158" s="256">
+      <c r="E158" s="188">
         <v>3.7</v>
       </c>
-      <c r="F158" s="256">
+      <c r="F158" s="188">
         <v>1.4</v>
       </c>
-      <c r="G158" s="256">
+      <c r="G158" s="188">
         <v>23.6</v>
       </c>
-      <c r="H158" s="256">
+      <c r="H158" s="188">
         <v>70.5</v>
       </c>
-      <c r="I158" s="256">
+      <c r="I158" s="188">
         <v>0.8</v>
       </c>
-      <c r="J158" s="257">
+      <c r="J158" s="189">
         <v>5.0999999999999996</v>
       </c>
-      <c r="K158" s="257">
+      <c r="K158" s="189">
         <v>94.1</v>
       </c>
-      <c r="L158" s="258">
+      <c r="L158" s="190">
         <v>3.6</v>
       </c>
-      <c r="M158" s="259">
+      <c r="M158" s="191">
         <v>0.7</v>
       </c>
     </row>
@@ -37029,16 +37037,16 @@
       <c r="I159" s="48">
         <v>7.7</v>
       </c>
-      <c r="J159" s="234">
+      <c r="J159" s="169">
         <v>24.7</v>
       </c>
-      <c r="K159" s="234">
+      <c r="K159" s="169">
         <v>67.7</v>
       </c>
-      <c r="L159" s="235">
+      <c r="L159" s="170">
         <v>3</v>
       </c>
-      <c r="M159" s="260">
+      <c r="M159" s="192">
         <v>0.99</v>
       </c>
     </row>
@@ -37065,16 +37073,16 @@
       <c r="I160" s="44">
         <v>6.8</v>
       </c>
-      <c r="J160" s="236">
+      <c r="J160" s="171">
         <v>69.2</v>
       </c>
-      <c r="K160" s="236">
+      <c r="K160" s="171">
         <v>24.1</v>
       </c>
-      <c r="L160" s="237">
+      <c r="L160" s="172">
         <v>1.9</v>
       </c>
-      <c r="M160" s="255">
+      <c r="M160" s="187">
         <v>1.02</v>
       </c>
     </row>
@@ -37085,34 +37093,34 @@
       <c r="C161" s="50" t="s">
         <v>277</v>
       </c>
-      <c r="D161" s="256">
+      <c r="D161" s="188">
         <v>-1059</v>
       </c>
-      <c r="E161" s="256">
+      <c r="E161" s="188">
         <v>2.2999999999999998</v>
       </c>
-      <c r="F161" s="256">
+      <c r="F161" s="188">
         <v>0.7</v>
       </c>
-      <c r="G161" s="256">
+      <c r="G161" s="188">
         <v>29.3</v>
       </c>
-      <c r="H161" s="256">
+      <c r="H161" s="188">
         <v>66.5</v>
       </c>
-      <c r="I161" s="256">
+      <c r="I161" s="188">
         <v>1.2</v>
       </c>
-      <c r="J161" s="257">
+      <c r="J161" s="189">
         <v>3</v>
       </c>
-      <c r="K161" s="257">
+      <c r="K161" s="189">
         <v>95.8</v>
       </c>
-      <c r="L161" s="258">
+      <c r="L161" s="190">
         <v>3.6</v>
       </c>
-      <c r="M161" s="259">
+      <c r="M161" s="191">
         <v>0.62</v>
       </c>
     </row>
@@ -37141,16 +37149,16 @@
       <c r="I162" s="48">
         <v>7.7</v>
       </c>
-      <c r="J162" s="234">
+      <c r="J162" s="169">
         <v>77.2</v>
       </c>
-      <c r="K162" s="234">
+      <c r="K162" s="169">
         <v>15.1</v>
       </c>
-      <c r="L162" s="235">
+      <c r="L162" s="170">
         <v>1.7</v>
       </c>
-      <c r="M162" s="260">
+      <c r="M162" s="192">
         <v>0.78</v>
       </c>
     </row>
@@ -37177,16 +37185,16 @@
       <c r="I163" s="48">
         <v>3</v>
       </c>
-      <c r="J163" s="234">
+      <c r="J163" s="169">
         <v>1.6</v>
       </c>
-      <c r="K163" s="234">
+      <c r="K163" s="169">
         <v>95.4</v>
       </c>
-      <c r="L163" s="235">
+      <c r="L163" s="170">
         <v>3.6</v>
       </c>
-      <c r="M163" s="260">
+      <c r="M163" s="192">
         <v>0.55000000000000004</v>
       </c>
     </row>
@@ -37213,16 +37221,16 @@
       <c r="I164" s="48">
         <v>10.9</v>
       </c>
-      <c r="J164" s="234">
+      <c r="J164" s="169">
         <v>0</v>
       </c>
-      <c r="K164" s="234">
+      <c r="K164" s="169">
         <v>89.1</v>
       </c>
-      <c r="L164" s="235">
+      <c r="L164" s="170">
         <v>3.2</v>
       </c>
-      <c r="M164" s="260">
+      <c r="M164" s="192">
         <v>0.42</v>
       </c>
     </row>
@@ -37249,16 +37257,16 @@
       <c r="I165" s="48">
         <v>11.4</v>
       </c>
-      <c r="J165" s="234">
+      <c r="J165" s="169">
         <v>49</v>
       </c>
-      <c r="K165" s="234">
+      <c r="K165" s="169">
         <v>39.5</v>
       </c>
-      <c r="L165" s="235">
+      <c r="L165" s="170">
         <v>2.2999999999999998</v>
       </c>
-      <c r="M165" s="260">
+      <c r="M165" s="192">
         <v>0.8</v>
       </c>
     </row>
@@ -37285,16 +37293,16 @@
       <c r="I166" s="48">
         <v>4</v>
       </c>
-      <c r="J166" s="234">
+      <c r="J166" s="169">
         <v>52.8</v>
       </c>
-      <c r="K166" s="234">
+      <c r="K166" s="169">
         <v>43.2</v>
       </c>
-      <c r="L166" s="235">
+      <c r="L166" s="170">
         <v>2.1</v>
       </c>
-      <c r="M166" s="260">
+      <c r="M166" s="192">
         <v>1.27</v>
       </c>
     </row>
@@ -37321,16 +37329,16 @@
       <c r="I167" s="48">
         <v>19.600000000000001</v>
       </c>
-      <c r="J167" s="234">
+      <c r="J167" s="169">
         <v>37.9</v>
       </c>
-      <c r="K167" s="234">
+      <c r="K167" s="169">
         <v>42.5</v>
       </c>
-      <c r="L167" s="235">
+      <c r="L167" s="170">
         <v>2.2999999999999998</v>
       </c>
-      <c r="M167" s="260">
+      <c r="M167" s="192">
         <v>0.86</v>
       </c>
       <c r="O167">
@@ -37361,31 +37369,33 @@
       <c r="I168" s="44">
         <v>17.600000000000001</v>
       </c>
-      <c r="J168" s="236">
+      <c r="J168" s="171">
         <v>34.200000000000003</v>
       </c>
-      <c r="K168" s="236">
+      <c r="K168" s="171">
         <v>48.3</v>
       </c>
-      <c r="L168" s="237">
+      <c r="L168" s="172">
         <v>2.4</v>
       </c>
-      <c r="M168" s="255">
+      <c r="M168" s="187">
         <v>0.88</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="M139:M141"/>
-    <mergeCell ref="B142:C142"/>
-    <mergeCell ref="B143:B144"/>
-    <mergeCell ref="B145:B150"/>
-    <mergeCell ref="B151:B157"/>
-    <mergeCell ref="B139:C141"/>
-    <mergeCell ref="D139:D141"/>
-    <mergeCell ref="J139:J141"/>
-    <mergeCell ref="K139:K141"/>
-    <mergeCell ref="L139:L141"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A11"/>
+    <mergeCell ref="A12:A18"/>
+    <mergeCell ref="L102:R102"/>
+    <mergeCell ref="S102:U102"/>
+    <mergeCell ref="B105:B106"/>
+    <mergeCell ref="D102:E102"/>
+    <mergeCell ref="C84:C86"/>
+    <mergeCell ref="C87:C94"/>
     <mergeCell ref="C110:C111"/>
     <mergeCell ref="C112:C117"/>
     <mergeCell ref="C118:C124"/>
@@ -37400,18 +37410,16 @@
     <mergeCell ref="C69:C70"/>
     <mergeCell ref="C71:C76"/>
     <mergeCell ref="C77:C83"/>
-    <mergeCell ref="L102:R102"/>
-    <mergeCell ref="S102:U102"/>
-    <mergeCell ref="B105:B106"/>
-    <mergeCell ref="D102:E102"/>
-    <mergeCell ref="C84:C86"/>
-    <mergeCell ref="C87:C94"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A11"/>
-    <mergeCell ref="A12:A18"/>
+    <mergeCell ref="M139:M141"/>
+    <mergeCell ref="B142:C142"/>
+    <mergeCell ref="B143:B144"/>
+    <mergeCell ref="B145:B150"/>
+    <mergeCell ref="B151:B157"/>
+    <mergeCell ref="B139:C141"/>
+    <mergeCell ref="D139:D141"/>
+    <mergeCell ref="J139:J141"/>
+    <mergeCell ref="K139:K141"/>
+    <mergeCell ref="L139:L141"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="G68:G94">
@@ -37617,8 +37625,8 @@
     </row>
     <row r="3" spans="4:10" ht="21">
       <c r="D3" s="115"/>
-      <c r="E3" s="217"/>
-      <c r="F3" s="217"/>
+      <c r="E3" s="267"/>
+      <c r="F3" s="267"/>
       <c r="G3" s="131" t="s">
         <v>225</v>
       </c>
@@ -37632,10 +37640,10 @@
     </row>
     <row r="4" spans="4:10" ht="12" customHeight="1">
       <c r="D4" s="115"/>
-      <c r="E4" s="218" t="s">
+      <c r="E4" s="268" t="s">
         <v>82</v>
       </c>
-      <c r="F4" s="218"/>
+      <c r="F4" s="268"/>
       <c r="G4" s="132">
         <v>49.3</v>
       </c>
@@ -37649,7 +37657,7 @@
     </row>
     <row r="5" spans="4:10" ht="12" customHeight="1">
       <c r="D5" s="115"/>
-      <c r="E5" s="216" t="s">
+      <c r="E5" s="266" t="s">
         <v>83</v>
       </c>
       <c r="F5" s="134" t="s">
@@ -37668,7 +37676,7 @@
     </row>
     <row r="6" spans="4:10" ht="12" customHeight="1">
       <c r="D6" s="115"/>
-      <c r="E6" s="216"/>
+      <c r="E6" s="266"/>
       <c r="F6" s="134" t="s">
         <v>85</v>
       </c>
@@ -37685,7 +37693,7 @@
     </row>
     <row r="7" spans="4:10" ht="12" customHeight="1">
       <c r="D7" s="115"/>
-      <c r="E7" s="216" t="s">
+      <c r="E7" s="266" t="s">
         <v>86</v>
       </c>
       <c r="F7" s="134" t="s">
@@ -37704,7 +37712,7 @@
     </row>
     <row r="8" spans="4:10" ht="12" customHeight="1">
       <c r="D8" s="115"/>
-      <c r="E8" s="216"/>
+      <c r="E8" s="266"/>
       <c r="F8" s="134" t="s">
         <v>128</v>
       </c>
@@ -37721,7 +37729,7 @@
     </row>
     <row r="9" spans="4:10" ht="12" customHeight="1">
       <c r="D9" s="115"/>
-      <c r="E9" s="216"/>
+      <c r="E9" s="266"/>
       <c r="F9" s="134" t="s">
         <v>129</v>
       </c>
@@ -37738,7 +37746,7 @@
     </row>
     <row r="10" spans="4:10" ht="12" customHeight="1">
       <c r="D10" s="115"/>
-      <c r="E10" s="216"/>
+      <c r="E10" s="266"/>
       <c r="F10" s="134" t="s">
         <v>130</v>
       </c>
@@ -37755,7 +37763,7 @@
     </row>
     <row r="11" spans="4:10" ht="12" customHeight="1">
       <c r="D11" s="115"/>
-      <c r="E11" s="216"/>
+      <c r="E11" s="266"/>
       <c r="F11" s="134" t="s">
         <v>131</v>
       </c>
@@ -37772,7 +37780,7 @@
     </row>
     <row r="12" spans="4:10" ht="12" customHeight="1">
       <c r="D12" s="115"/>
-      <c r="E12" s="216"/>
+      <c r="E12" s="266"/>
       <c r="F12" s="134" t="s">
         <v>132</v>
       </c>
@@ -37789,7 +37797,7 @@
     </row>
     <row r="13" spans="4:10" ht="12" customHeight="1">
       <c r="D13" s="115"/>
-      <c r="E13" s="216" t="s">
+      <c r="E13" s="266" t="s">
         <v>139</v>
       </c>
       <c r="F13" s="134" t="s">
@@ -37808,7 +37816,7 @@
     </row>
     <row r="14" spans="4:10" ht="12" customHeight="1">
       <c r="D14" s="115"/>
-      <c r="E14" s="216"/>
+      <c r="E14" s="266"/>
       <c r="F14" s="134" t="s">
         <v>114</v>
       </c>
@@ -37825,7 +37833,7 @@
     </row>
     <row r="15" spans="4:10" ht="12" customHeight="1">
       <c r="D15" s="115"/>
-      <c r="E15" s="216"/>
+      <c r="E15" s="266"/>
       <c r="F15" s="134" t="s">
         <v>148</v>
       </c>
@@ -37842,7 +37850,7 @@
     </row>
     <row r="16" spans="4:10" ht="12" customHeight="1">
       <c r="D16" s="115"/>
-      <c r="E16" s="216"/>
+      <c r="E16" s="266"/>
       <c r="F16" s="134" t="s">
         <v>117</v>
       </c>
@@ -37859,7 +37867,7 @@
     </row>
     <row r="17" spans="4:10" ht="12" customHeight="1">
       <c r="D17" s="115"/>
-      <c r="E17" s="216"/>
+      <c r="E17" s="266"/>
       <c r="F17" s="134" t="s">
         <v>119</v>
       </c>
@@ -37876,7 +37884,7 @@
     </row>
     <row r="18" spans="4:10" ht="12" customHeight="1">
       <c r="D18" s="115"/>
-      <c r="E18" s="216"/>
+      <c r="E18" s="266"/>
       <c r="F18" s="134" t="s">
         <v>121</v>
       </c>
@@ -37893,7 +37901,7 @@
     </row>
     <row r="19" spans="4:10" ht="12" customHeight="1">
       <c r="D19" s="115"/>
-      <c r="E19" s="216"/>
+      <c r="E19" s="266"/>
       <c r="F19" s="134" t="s">
         <v>123</v>
       </c>
@@ -37910,7 +37918,7 @@
     </row>
     <row r="20" spans="4:10" ht="12" customHeight="1">
       <c r="D20" s="115"/>
-      <c r="E20" s="216" t="s">
+      <c r="E20" s="266" t="s">
         <v>111</v>
       </c>
       <c r="F20" s="134" t="s">
@@ -37929,7 +37937,7 @@
     </row>
     <row r="21" spans="4:10" ht="12" customHeight="1">
       <c r="D21" s="115"/>
-      <c r="E21" s="216"/>
+      <c r="E21" s="266"/>
       <c r="F21" s="134" t="s">
         <v>35</v>
       </c>
@@ -37946,7 +37954,7 @@
     </row>
     <row r="22" spans="4:10" ht="12" customHeight="1">
       <c r="D22" s="115"/>
-      <c r="E22" s="216"/>
+      <c r="E22" s="266"/>
       <c r="F22" s="134" t="s">
         <v>36</v>
       </c>
@@ -37963,7 +37971,7 @@
     </row>
     <row r="23" spans="4:10" ht="12" customHeight="1">
       <c r="D23" s="115"/>
-      <c r="E23" s="216" t="s">
+      <c r="E23" s="266" t="s">
         <v>112</v>
       </c>
       <c r="F23" s="134" t="s">
@@ -37982,7 +37990,7 @@
     </row>
     <row r="24" spans="4:10" ht="12" customHeight="1">
       <c r="D24" s="115"/>
-      <c r="E24" s="216"/>
+      <c r="E24" s="266"/>
       <c r="F24" s="134" t="s">
         <v>27</v>
       </c>
@@ -37999,7 +38007,7 @@
     </row>
     <row r="25" spans="4:10" ht="12" customHeight="1">
       <c r="D25" s="115"/>
-      <c r="E25" s="216"/>
+      <c r="E25" s="266"/>
       <c r="F25" s="134" t="s">
         <v>28</v>
       </c>
@@ -38016,7 +38024,7 @@
     </row>
     <row r="26" spans="4:10" ht="12" customHeight="1">
       <c r="D26" s="115"/>
-      <c r="E26" s="216"/>
+      <c r="E26" s="266"/>
       <c r="F26" s="134" t="s">
         <v>30</v>
       </c>
@@ -38033,7 +38041,7 @@
     </row>
     <row r="27" spans="4:10" ht="12" customHeight="1">
       <c r="D27" s="115"/>
-      <c r="E27" s="216"/>
+      <c r="E27" s="266"/>
       <c r="F27" s="134" t="s">
         <v>29</v>
       </c>
@@ -38050,7 +38058,7 @@
     </row>
     <row r="28" spans="4:10" ht="12" customHeight="1">
       <c r="D28" s="115"/>
-      <c r="E28" s="216"/>
+      <c r="E28" s="266"/>
       <c r="F28" s="134" t="s">
         <v>105</v>
       </c>
@@ -38067,7 +38075,7 @@
     </row>
     <row r="29" spans="4:10" ht="12" customHeight="1">
       <c r="D29" s="115"/>
-      <c r="E29" s="216"/>
+      <c r="E29" s="266"/>
       <c r="F29" s="134" t="s">
         <v>106</v>
       </c>
@@ -38084,7 +38092,7 @@
     </row>
     <row r="30" spans="4:10" ht="12" customHeight="1">
       <c r="D30" s="115"/>
-      <c r="E30" s="216"/>
+      <c r="E30" s="266"/>
       <c r="F30" s="134" t="s">
         <v>55</v>
       </c>
@@ -38108,8 +38116,8 @@
     </row>
     <row r="32" spans="4:10" ht="21">
       <c r="D32" s="115"/>
-      <c r="E32" s="217"/>
-      <c r="F32" s="217"/>
+      <c r="E32" s="267"/>
+      <c r="F32" s="267"/>
       <c r="G32" s="131" t="s">
         <v>225</v>
       </c>
@@ -38123,10 +38131,10 @@
     </row>
     <row r="33" spans="4:10" ht="12" customHeight="1">
       <c r="D33" s="115"/>
-      <c r="E33" s="218" t="s">
+      <c r="E33" s="268" t="s">
         <v>82</v>
       </c>
-      <c r="F33" s="218"/>
+      <c r="F33" s="268"/>
       <c r="G33" s="132">
         <v>49.3</v>
       </c>
@@ -38140,7 +38148,7 @@
     </row>
     <row r="34" spans="4:10" ht="12" customHeight="1">
       <c r="D34" s="115"/>
-      <c r="E34" s="216" t="s">
+      <c r="E34" s="266" t="s">
         <v>83</v>
       </c>
       <c r="F34" s="134" t="s">
@@ -38159,7 +38167,7 @@
     </row>
     <row r="35" spans="4:10" ht="12" customHeight="1">
       <c r="D35" s="115"/>
-      <c r="E35" s="216"/>
+      <c r="E35" s="266"/>
       <c r="F35" s="134" t="s">
         <v>85</v>
       </c>
@@ -38176,7 +38184,7 @@
     </row>
     <row r="36" spans="4:10" ht="12" customHeight="1">
       <c r="D36" s="115"/>
-      <c r="E36" s="216" t="s">
+      <c r="E36" s="266" t="s">
         <v>86</v>
       </c>
       <c r="F36" s="134" t="s">
@@ -38195,7 +38203,7 @@
     </row>
     <row r="37" spans="4:10" ht="12" customHeight="1">
       <c r="D37" s="115"/>
-      <c r="E37" s="216"/>
+      <c r="E37" s="266"/>
       <c r="F37" s="134" t="s">
         <v>128</v>
       </c>
@@ -38212,7 +38220,7 @@
     </row>
     <row r="38" spans="4:10" ht="12" customHeight="1">
       <c r="D38" s="115"/>
-      <c r="E38" s="216"/>
+      <c r="E38" s="266"/>
       <c r="F38" s="134" t="s">
         <v>129</v>
       </c>
@@ -38229,7 +38237,7 @@
     </row>
     <row r="39" spans="4:10" ht="12" customHeight="1">
       <c r="D39" s="115"/>
-      <c r="E39" s="216"/>
+      <c r="E39" s="266"/>
       <c r="F39" s="134" t="s">
         <v>130</v>
       </c>
@@ -38246,7 +38254,7 @@
     </row>
     <row r="40" spans="4:10" ht="12" customHeight="1">
       <c r="D40" s="115"/>
-      <c r="E40" s="216"/>
+      <c r="E40" s="266"/>
       <c r="F40" s="134" t="s">
         <v>131</v>
       </c>
@@ -38263,7 +38271,7 @@
     </row>
     <row r="41" spans="4:10" ht="12" customHeight="1">
       <c r="D41" s="115"/>
-      <c r="E41" s="216"/>
+      <c r="E41" s="266"/>
       <c r="F41" s="134" t="s">
         <v>132</v>
       </c>
@@ -38280,7 +38288,7 @@
     </row>
     <row r="42" spans="4:10" ht="12" customHeight="1">
       <c r="D42" s="115"/>
-      <c r="E42" s="216" t="s">
+      <c r="E42" s="266" t="s">
         <v>139</v>
       </c>
       <c r="F42" s="134" t="s">
@@ -38299,7 +38307,7 @@
     </row>
     <row r="43" spans="4:10" ht="12" customHeight="1">
       <c r="D43" s="115"/>
-      <c r="E43" s="216"/>
+      <c r="E43" s="266"/>
       <c r="F43" s="134" t="s">
         <v>114</v>
       </c>
@@ -38316,7 +38324,7 @@
     </row>
     <row r="44" spans="4:10" ht="12" customHeight="1">
       <c r="D44" s="115"/>
-      <c r="E44" s="216"/>
+      <c r="E44" s="266"/>
       <c r="F44" s="134" t="s">
         <v>148</v>
       </c>
@@ -38333,7 +38341,7 @@
     </row>
     <row r="45" spans="4:10" ht="12" customHeight="1">
       <c r="D45" s="115"/>
-      <c r="E45" s="216"/>
+      <c r="E45" s="266"/>
       <c r="F45" s="134" t="s">
         <v>117</v>
       </c>
@@ -38350,7 +38358,7 @@
     </row>
     <row r="46" spans="4:10" ht="12" customHeight="1">
       <c r="D46" s="115"/>
-      <c r="E46" s="216"/>
+      <c r="E46" s="266"/>
       <c r="F46" s="134" t="s">
         <v>119</v>
       </c>
@@ -38367,7 +38375,7 @@
     </row>
     <row r="47" spans="4:10" ht="12" customHeight="1">
       <c r="D47" s="115"/>
-      <c r="E47" s="216"/>
+      <c r="E47" s="266"/>
       <c r="F47" s="134" t="s">
         <v>121</v>
       </c>
@@ -38384,7 +38392,7 @@
     </row>
     <row r="48" spans="4:10" ht="12" customHeight="1">
       <c r="D48" s="115"/>
-      <c r="E48" s="216"/>
+      <c r="E48" s="266"/>
       <c r="F48" s="134" t="s">
         <v>123</v>
       </c>
@@ -38401,7 +38409,7 @@
     </row>
     <row r="49" spans="2:10" ht="12" customHeight="1">
       <c r="D49" s="115"/>
-      <c r="E49" s="216" t="s">
+      <c r="E49" s="266" t="s">
         <v>111</v>
       </c>
       <c r="F49" s="134" t="s">
@@ -38420,7 +38428,7 @@
     </row>
     <row r="50" spans="2:10" ht="12" customHeight="1">
       <c r="D50" s="115"/>
-      <c r="E50" s="216"/>
+      <c r="E50" s="266"/>
       <c r="F50" s="134" t="s">
         <v>35</v>
       </c>
@@ -38437,7 +38445,7 @@
     </row>
     <row r="51" spans="2:10" ht="12" customHeight="1">
       <c r="D51" s="115"/>
-      <c r="E51" s="216"/>
+      <c r="E51" s="266"/>
       <c r="F51" s="134" t="s">
         <v>36</v>
       </c>
@@ -38454,7 +38462,7 @@
     </row>
     <row r="52" spans="2:10" ht="12" customHeight="1">
       <c r="D52" s="115"/>
-      <c r="E52" s="216" t="s">
+      <c r="E52" s="266" t="s">
         <v>112</v>
       </c>
       <c r="F52" s="134" t="s">
@@ -38473,7 +38481,7 @@
     </row>
     <row r="53" spans="2:10" ht="12" customHeight="1">
       <c r="D53" s="115"/>
-      <c r="E53" s="216"/>
+      <c r="E53" s="266"/>
       <c r="F53" s="134" t="s">
         <v>27</v>
       </c>
@@ -38490,7 +38498,7 @@
     </row>
     <row r="54" spans="2:10" ht="12" customHeight="1">
       <c r="D54" s="115"/>
-      <c r="E54" s="216"/>
+      <c r="E54" s="266"/>
       <c r="F54" s="134" t="s">
         <v>28</v>
       </c>
@@ -38507,7 +38515,7 @@
     </row>
     <row r="55" spans="2:10" ht="12" customHeight="1">
       <c r="D55" s="115"/>
-      <c r="E55" s="216"/>
+      <c r="E55" s="266"/>
       <c r="F55" s="134" t="s">
         <v>30</v>
       </c>
@@ -38524,7 +38532,7 @@
     </row>
     <row r="56" spans="2:10" ht="12" customHeight="1">
       <c r="D56" s="115"/>
-      <c r="E56" s="216"/>
+      <c r="E56" s="266"/>
       <c r="F56" s="134" t="s">
         <v>29</v>
       </c>
@@ -38541,14 +38549,14 @@
     </row>
     <row r="57" spans="2:10" ht="12" customHeight="1">
       <c r="D57" s="115"/>
-      <c r="E57" s="216"/>
+      <c r="E57" s="266"/>
       <c r="F57" s="134" t="s">
         <v>105</v>
       </c>
-      <c r="G57" s="246">
+      <c r="G57" s="178">
         <v>24.9</v>
       </c>
-      <c r="H57" s="246">
+      <c r="H57" s="178">
         <v>46.4</v>
       </c>
       <c r="I57" s="137">
@@ -38558,14 +38566,14 @@
     </row>
     <row r="58" spans="2:10" ht="12" customHeight="1">
       <c r="D58" s="115"/>
-      <c r="E58" s="216"/>
+      <c r="E58" s="266"/>
       <c r="F58" s="134" t="s">
         <v>262</v>
       </c>
-      <c r="G58" s="246">
+      <c r="G58" s="178">
         <v>13.329743451206161</v>
       </c>
-      <c r="H58" s="246">
+      <c r="H58" s="178">
         <v>38.524030878104121</v>
       </c>
       <c r="I58" s="137">
@@ -38676,8 +38684,8 @@
     </row>
     <row r="97" spans="15:21" ht="21">
       <c r="O97" s="115"/>
-      <c r="P97" s="217"/>
-      <c r="Q97" s="217"/>
+      <c r="P97" s="267"/>
+      <c r="Q97" s="267"/>
       <c r="R97" s="131" t="s">
         <v>222</v>
       </c>
@@ -38691,7 +38699,7 @@
     </row>
     <row r="98" spans="15:21">
       <c r="O98" s="115"/>
-      <c r="P98" s="219" t="s">
+      <c r="P98" s="269" t="s">
         <v>83</v>
       </c>
       <c r="Q98" s="140" t="s">
@@ -38711,7 +38719,7 @@
     </row>
     <row r="99" spans="15:21">
       <c r="O99" s="115"/>
-      <c r="P99" s="219"/>
+      <c r="P99" s="269"/>
       <c r="Q99" s="140" t="s">
         <v>144</v>
       </c>
@@ -38729,7 +38737,7 @@
     </row>
     <row r="100" spans="15:21">
       <c r="O100" s="115"/>
-      <c r="P100" s="219" t="s">
+      <c r="P100" s="269" t="s">
         <v>138</v>
       </c>
       <c r="Q100" s="140" t="s">
@@ -38749,7 +38757,7 @@
     </row>
     <row r="101" spans="15:21">
       <c r="O101" s="115"/>
-      <c r="P101" s="219"/>
+      <c r="P101" s="269"/>
       <c r="Q101" s="140" t="s">
         <v>128</v>
       </c>
@@ -38767,7 +38775,7 @@
     </row>
     <row r="102" spans="15:21">
       <c r="O102" s="115"/>
-      <c r="P102" s="219"/>
+      <c r="P102" s="269"/>
       <c r="Q102" s="140" t="s">
         <v>129</v>
       </c>
@@ -38785,7 +38793,7 @@
     </row>
     <row r="103" spans="15:21">
       <c r="O103" s="115"/>
-      <c r="P103" s="219"/>
+      <c r="P103" s="269"/>
       <c r="Q103" s="140" t="s">
         <v>130</v>
       </c>
@@ -38803,7 +38811,7 @@
     </row>
     <row r="104" spans="15:21">
       <c r="O104" s="115"/>
-      <c r="P104" s="219"/>
+      <c r="P104" s="269"/>
       <c r="Q104" s="140" t="s">
         <v>131</v>
       </c>
@@ -38821,7 +38829,7 @@
     </row>
     <row r="105" spans="15:21">
       <c r="O105" s="115"/>
-      <c r="P105" s="219"/>
+      <c r="P105" s="269"/>
       <c r="Q105" s="140" t="s">
         <v>132</v>
       </c>
@@ -38839,7 +38847,7 @@
     </row>
     <row r="106" spans="15:21">
       <c r="O106" s="115"/>
-      <c r="P106" s="219" t="s">
+      <c r="P106" s="269" t="s">
         <v>139</v>
       </c>
       <c r="Q106" s="134" t="s">
@@ -38859,7 +38867,7 @@
     </row>
     <row r="107" spans="15:21">
       <c r="O107" s="115"/>
-      <c r="P107" s="219"/>
+      <c r="P107" s="269"/>
       <c r="Q107" s="134" t="s">
         <v>114</v>
       </c>
@@ -38877,7 +38885,7 @@
     </row>
     <row r="108" spans="15:21">
       <c r="O108" s="115"/>
-      <c r="P108" s="219"/>
+      <c r="P108" s="269"/>
       <c r="Q108" s="134" t="s">
         <v>148</v>
       </c>
@@ -38895,7 +38903,7 @@
     </row>
     <row r="109" spans="15:21">
       <c r="O109" s="115"/>
-      <c r="P109" s="219"/>
+      <c r="P109" s="269"/>
       <c r="Q109" s="134" t="s">
         <v>117</v>
       </c>
@@ -38913,7 +38921,7 @@
     </row>
     <row r="110" spans="15:21">
       <c r="O110" s="115"/>
-      <c r="P110" s="219"/>
+      <c r="P110" s="269"/>
       <c r="Q110" s="134" t="s">
         <v>119</v>
       </c>
@@ -38931,7 +38939,7 @@
     </row>
     <row r="111" spans="15:21">
       <c r="O111" s="115"/>
-      <c r="P111" s="219"/>
+      <c r="P111" s="269"/>
       <c r="Q111" s="134" t="s">
         <v>121</v>
       </c>
@@ -38949,7 +38957,7 @@
     </row>
     <row r="112" spans="15:21">
       <c r="O112" s="115"/>
-      <c r="P112" s="219"/>
+      <c r="P112" s="269"/>
       <c r="Q112" s="134" t="s">
         <v>123</v>
       </c>
@@ -38967,7 +38975,7 @@
     </row>
     <row r="113" spans="15:21">
       <c r="O113" s="115"/>
-      <c r="P113" s="219" t="s">
+      <c r="P113" s="269" t="s">
         <v>111</v>
       </c>
       <c r="Q113" s="140" t="s">
@@ -38987,7 +38995,7 @@
     </row>
     <row r="114" spans="15:21">
       <c r="O114" s="115"/>
-      <c r="P114" s="219"/>
+      <c r="P114" s="269"/>
       <c r="Q114" s="140" t="s">
         <v>35</v>
       </c>
@@ -39005,7 +39013,7 @@
     </row>
     <row r="115" spans="15:21">
       <c r="O115" s="115"/>
-      <c r="P115" s="219"/>
+      <c r="P115" s="269"/>
       <c r="Q115" s="140" t="s">
         <v>36</v>
       </c>
@@ -39030,6 +39038,18 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="E23:E30"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E12"/>
+    <mergeCell ref="E13:E19"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="P97:Q97"/>
+    <mergeCell ref="P98:P99"/>
+    <mergeCell ref="P100:P105"/>
+    <mergeCell ref="P106:P112"/>
+    <mergeCell ref="P113:P115"/>
     <mergeCell ref="E49:E51"/>
     <mergeCell ref="E52:E58"/>
     <mergeCell ref="E32:F32"/>
@@ -39037,18 +39057,6 @@
     <mergeCell ref="E34:E35"/>
     <mergeCell ref="E36:E41"/>
     <mergeCell ref="E42:E48"/>
-    <mergeCell ref="P97:Q97"/>
-    <mergeCell ref="P98:P99"/>
-    <mergeCell ref="P100:P105"/>
-    <mergeCell ref="P106:P112"/>
-    <mergeCell ref="P113:P115"/>
-    <mergeCell ref="E23:E30"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E7:E12"/>
-    <mergeCell ref="E13:E19"/>
-    <mergeCell ref="E20:E22"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="I4:I30">
@@ -39065,6 +39073,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I33:I58">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{50ACF02A-6109-45DB-A715-AF1FB70A1773}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="T98:T115">
     <cfRule type="dataBar" priority="2">
       <dataBar>
@@ -39075,20 +39097,6 @@
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{A4492945-8F85-41E2-9CC5-40C2647B42DB}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I33:I58">
-    <cfRule type="dataBar" priority="5">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50ACF02A-6109-45DB-A715-AF1FB70A1773}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -39113,6 +39121,19 @@
           <xm:sqref>I4:I30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{50ACF02A-6109-45DB-A715-AF1FB70A1773}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I33:I58</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{A4492945-8F85-41E2-9CC5-40C2647B42DB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -39124,19 +39145,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>T98:T115</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50ACF02A-6109-45DB-A715-AF1FB70A1773}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I33:I58</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -40603,14 +40611,14 @@
       </c>
     </row>
     <row r="46" spans="4:10" ht="19.5">
-      <c r="D46" s="220" t="s">
+      <c r="D46" s="270" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="220"/>
-      <c r="F46" s="221" t="s">
+      <c r="E46" s="270"/>
+      <c r="F46" s="271" t="s">
         <v>141</v>
       </c>
-      <c r="G46" s="221"/>
+      <c r="G46" s="271"/>
     </row>
     <row r="47" spans="4:10">
       <c r="D47" s="162" t="s">
@@ -40919,6 +40927,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x0101009F70DF5EB7229D43B07112227358BB1E" ma:contentTypeVersion="12" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="22c22a957ab1dee50b95c413389aad32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b066b759-8662-4812-be3e-757f1ad2293d" xmlns:ns3="ede0981e-caa1-4e34-b056-7cb7259069de" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="99271caf908136a0b031c32453db0c57" ns2:_="" ns3:_="">
     <xsd:import namespace="b066b759-8662-4812-be3e-757f1ad2293d"/>
@@ -41119,15 +41136,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -41140,6 +41148,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{721DA890-72B7-4FCC-BE33-9222AFCD9D13}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17BC2868-5334-4509-A134-C97C48625768}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41158,14 +41174,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{721DA890-72B7-4FCC-BE33-9222AFCD9D13}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{34D80DAD-C8C7-4AFF-8C59-F419E6E4993D}">
   <ds:schemaRefs>

</xml_diff>